<commit_message>
Il tuo messaggio di commit
</commit_message>
<xml_diff>
--- a/output/startup_estratte.xlsx
+++ b/output/startup_estratte.xlsx
@@ -906,17 +906,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>IT01038800148</t>
+          <t>IT00977110949</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>WIDE VR S.R.L.</t>
+          <t>MEDITERRANEA SOCIETA' A RESPONSABILITA' LIMITATA SEMPLIFICATA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>WIDE VR</t>
+          <t>MEDITERRANEA</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -926,22 +926,22 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>MILANO (MI)</t>
+          <t>ISERNIA (IS)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>MI</t>
+          <t>IS</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>LOMBARDIA</t>
+          <t>MOLISE</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>SOCIETA' A RESPONSABILITA' LIMITATA</t>
+          <t>SOCIETA' A RESPONSABILITA' LIMITATA SEMPLIFICATA</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>www.widevr.eu</t>
+          <t>www.mediterranea-lide.com</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>edoardo@widevr.eu</t>
+          <t>studio.mediterrranea@gmail.com</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -971,341 +971,520 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>https://startup.registroimprese.it/isin/dettaglioStartup?id=KXU3bCJQBfS92AJOXqJVKg%2BWN%2BjuDCsqwKwmUQbhow%3D%3D</t>
+          <t>https://startup.registroimprese.it/isin/dettaglioStartup?id=KXU3bCJQBfS92AJOXqJVKg%2BWN%2BnnCCQjwawuUQfhow%3D%3D</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>629009</t>
+          <t>439909</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
+          <t>Costruzione di piscine ed altri lavori specializzati di costruzione nca</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>INDUSTRIA/ARTIGIANATO</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>MS10</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Servizi</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>architettura, Antisismico, Ingegneria</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>16/01/2020</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>09/07/2020</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>18/06/2024</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>non disponibile</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>non disponibile</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>Non disponibile</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>Non disponibile</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>Non disponibile</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>SÌ</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>SÌ</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>SÌ</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>PIER LUIGI PACITTI</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>18/06/2024</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>InfoCamere Qualified Electronic Signature CA</t>
+        </is>
+      </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>00977110949-20240618173252</t>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>https://i.ibb.co/gFW3sFxK/67041bd45529.jpg</t>
+        </is>
+      </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>Disponibile (Caricato su ImgBB)</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
           <t>NON RILEVATO</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>SERVIZI</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>MS9</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>E-commerce</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>RealtaVirtuale</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>06/03/2020</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>12/01/2023</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
+      <c r="AR2" t="inlineStr">
         <is>
           <t>NON RILEVATO</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>14/10/2025</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>100K-500K euro</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>100K-500K euro</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="AE2" t="inlineStr">
-        <is>
-          <t>Non disponibile</t>
-        </is>
-      </c>
-      <c r="AF2" t="inlineStr">
-        <is>
-          <t>Non disponibile</t>
-        </is>
-      </c>
-      <c r="AG2" t="inlineStr">
-        <is>
-          <t>Non disponibile</t>
-        </is>
-      </c>
-      <c r="AH2" t="inlineStr">
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>NON RILEVATO</t>
+        </is>
+      </c>
+      <c r="AT2" t="inlineStr">
+        <is>
+          <t>NON RILEVATO</t>
+        </is>
+      </c>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t>NON RILEVATO</t>
+        </is>
+      </c>
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>NON RILEVATO</t>
+        </is>
+      </c>
+      <c r="AW2" t="inlineStr">
+        <is>
+          <t>NON RILEVATO</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>NON RILEVATO</t>
+        </is>
+      </c>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="AZ2" t="inlineStr">
+        <is>
+          <t>Sviluppo</t>
+        </is>
+      </c>
+      <c r="BA2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="BB2" t="inlineStr">
+        <is>
+          <t>Prototipo/versione beta</t>
+        </is>
+      </c>
+      <c r="BC2" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="BD2" t="inlineStr">
+        <is>
+          <t>Completo solo lato tecnico</t>
+        </is>
+      </c>
+      <c r="BE2" t="inlineStr">
+        <is>
+          <t>Presentazione aziendale e delle attività correlate
+La società Mediterranea s.r.l.s., startup innovativa, licenziataria di brevetto per invenzione industriale G.A.E (Giunto Antisismico Elastomerico) componente fondamentale del sistema LE.A.D. (LEgature Antisismiche Dissipative), ha iniziato l’attività in data 16/01/2020.
+L’oggetto sociale consiste in lavorazioni specializzate su edifici in acciaio, cemento armato e muratura.
+Nello specifico, le lavorazioni consistono in un sistema strutturale di legatura di strutture civile intelaiate in acciaio, c.l.s armato e muratura (LE.A.D.), che permette di modificare e migliorare o adeguare la risposta dell'organismo strutturale in caso di sisma.
+Tutto il sistema è imperniato sulla realizzazione di controventi "dissipativi" costituiti da tiranti collegati attraverso Giunti Antisismici Elastomerici G.A.E. alla struttura portante, tali giunti hanno capacità di dissipare energia.
+La particolarità dell'invenzione consiste nella adozione dei predetti giunti, definiti "Giunti Antisismici Elastomerici" (GAE), ad elevata standardizzazione per consentirne il montaggio, in tempi estremamente rapidi, in una grande varietà di configurazioni geometriche sulle strutture portanti di un edificio, in modo da adeguare le strutture ai dettami della vigente normativa sismica nazionale.
+La Mediterranea s.r.l.s avrà come scopo lo sviluppo, la produzione e la commercializzazione e l’installazione del sistema LE.A.D. di cui il giunto elastomerico G.A.E. oggetto del brevetto è parte essenziale.
+La società Mediterranea, è composta da: Arch. Pier Luigi Pacitti,  Ing. Antonio Libero Bucci.
+L’Arch. Pier Luigi Pacitti e l’Ing. Antonio Libero Bucci hanno maturato una profonda esperienza nel campo tecnico, con particolare riguardo nel campo della progettazione architettonica e della ristrutturazione antisismica degli edifici, per i metodi di catalogazione e rilievo di detrattori ambientali e di verifica di strumenti urbanistici.
+Si evidenzia, nello specifico, l’ultraventennale esperienza acquisita nel campo procedurale con particolare riguardo per quel che riguarda l'iter burocratico/amministrativo delle pratiche progettuali, dalle autorizzazioni, alle leggi ambientali, urbanistiche, sul risparmio energetico, antisismiche, tecnologiche ed elettriche.
+L’Ing. Antonio Libero Bucci contitolare del brevetto e coinventore del sistema antisismico, laureatosi in Ingegneria Civile Edile presso l’Università degli Studi di Roma La Sapienza nel Luglio 1987, con esperienza trentennale nel campo della ristrutturazione edilizia , con particolare attività nel campo dell’adeguamento e
+miglioramento sismico degli edifici Il sistema di legature antisismiche dissipative si basa sulla realizzazione di legature a
+controventi "dissipativi" costituiti da tiranti collegati alla struttura attraverso particolari giunti che hanno la capacità di dissipare energia grazie ad elementi in
+elastomero.
+Mediterrranea S.r.L.s. Viale dei Pentri 117/a 86170 Isernia (IS)
+Viale dei Pentri 117/a 86170 Isernia tel/fax 0865 299759 – p.iva 00977110949
+studio.mediterrranea@gmail.com www.mediterrenea-lide.com
+V/2-2022</t>
+        </is>
+      </c>
+      <c r="BF2" t="inlineStr">
+        <is>
+          <t>Presentation of the company and related activities
+The company Mediterranea s.r.l.s., innovative startup, patent licensee for industrial invention G.A.E (Elastomeric Seismic Joint), fundamental component of the LE.A.D. (Dissipative Seismic Bindings), started the activity on 16/01/2020.
+The corporate purpose consists of specialized work on buildings in steel, reinforced concrete and masonry.
+Specifically, the processes consist of a structural system of ligation of civil structures framed in steel, reinforced concrete and masonry (LE.A.D.), which allows to modify and improve or adapt the response of the structural organism in the event of an earthquake.
+The whole system is based on the creation of "dissipative" bracing consisting of tie rods connected through G.A.E. to the supporting structure, these joints have the ability to dissipate energy.
+The particularity of the invention consists in the adoption of the aforementioned joints, defined as "Elastomeric Anti-Seismic Joints" (GAE), with high standardization to allow their assembly, in extremely short times, in a great variety of geometric configurations on the load-bearing structures of a building, in in order to adapt the structures to the dictates of the current national seismic legislation.
+Mediterranea s.r.l.s will have as its purpose the development, production and marketing and installation of the LE.A.D. of which the elastomeric joint G.A.E. the subject of the patent is an essential part.
+The Mediterranea company is composed of: Arch. Pier Luigi Pacitti, Ing. Antonio Libero Bucci.
+Arch. Pier Luigi Pacitti and Eng. Antonio Libero Bucci have gained a deep experience in the technical field, with particular regard in the field of architectural design and anti-seismic renovation of buildings, for the methods of cataloging and survey of environmental detractors and of verification of urban planning tools.
+Specifically, the over twenty years of experience acquired in the procedural field is highlighted with particular regard to the bureaucratic / administrative process of design practices, from authorizations, to environmental, urban planning, energy saving, anti-seismic, technological and electrical laws.
+Eng. Antonio Libero Bucci, co-owner of the patent and co-inventor of the anti-seismic system, graduated in Civil Engineering from the University of Rome La Sapienza in July 1987, with thirty years of experience in the field of building renovation, with particular activity in the field of adaptation and
+seismic improvement of buildings The system of anti-seismic dissipative ties is based on the realization of a
+"dissipative" bracing consisting of tie rods connected to the structure through special joints that have the ability to dissipate energy thanks to elements in
+elastomer.
+Mediterrranea S.r.L.s. Viale dei Pentri 117 / a 86170 Isernia (IS)
+Viale dei Pentri 117 / a 86170 Isernia tel / fax 0865 299759 - VAT number 00977110949
+studio.mediterrranea@gmail.com www.mediterrenea-lide.com
+V / 2-2022</t>
+        </is>
+      </c>
+      <c r="BG2" t="inlineStr">
+        <is>
+          <t>La particolarità dell'invenzione consiste proprio nell’adozione dei predetti giunti, denominati giunti antisismici con elastomeri (indicato dall'acronimo “GAE”).
+Tale giunto presenta elevata standardizzazione per consentirne il montaggio in tempi estremamente rapidi, in una grande varietà di configurazioni geometriche delle strutture portanti di un edificio.
+Il GAE è costituito da uno snodo cilindrico, appositamente concepito, che ospita la testa di tesatura di un tirante in barra filettata. L’adozione di barre filettate permette di contenere al minimo l’ingombro del sistema di serraggio e permette, tramite il semplice avvitamento di un dado, di conferire un pretensionamento del tirante, che verrà calibrato tramite chiavi dinamometriche. Il sistema di alloggiamento della testa tirante prevede l’interposizione di un elemento elastomerico di tipo Newton a caratterizzazione elasto-plastica, che conferisce la capacità di dissipare energia.
+Andando a dosare il pretensionamento del tirante e la risposta elastica della cartuccia di elastomero alloggiata nel giunto si riesce a “modulare” la reazione del tirante ed a “pilotare” la risposta in condizioni sismiche dell’intera struttura portante dell’edificio.
+In sintesi le caratteristiche del GAE sono:
+1. Capacità dissipativa modificabile in funzione delle necessità;
+2. Facilità di montaggio
+3. Facilità ed economicità di ripristino a seguito di sisma e di manutenzione periodica, grazie alla sostituibilità del solo elemento elastomerico alloggiato nel giunto (cartuccia);
+4. Dimensioni e peso contenuti per un agevole trasporto e montaggio;
+5. Ridotti tempi di montaggio.
+Per la valorizzazione della tecnologia brevettuale devono essere intrapresi studi analitici allo scopo di validare e perseguire miglioramenti del sistema; sono state individuate le tappe obbligatorie dello sviluppo prototipale necessarie alla vidimazione del sistema stesso da parte del Consiglio Superiore dei Lavori Pubblici.
+La società è beneficiaria del finanziamento di Euro 131.742,88 ottenuto attraverso il bando europeo BREVETTI+ finanziamento concesso da INVITALIA azienda nazionale per l’attrazione degli investimenti e lo sviluppo d’impresa SPA.
+Passaggio chiave dell’iter procedurale sarà, la realizzazione di un prototipo sperimentale, testato su tavola vibrante e analizzato in modo da procedere alla modellizzazione.
+Quindi, i servizi necessari allo sviluppo e alla successiva validazione del sistema sono:
+1) Analisi e industrializzazione dell’apparecchio, che include:
+a) Studio, progettazione ed ingegnerizzazione del prototipo:
+i) Modellazione e ingegnerizzazione;
+ii) Analisi statiche e dinamiche modellistiche sul dispositivo;
+iii) Analisi effetti dissipativi;
+iv) Analisi del filtraggio delle frequenze
+v) Analisi delle curve di isteresi e della capacità dissipativa dell’apparecchio
+vi) Analisi dei fattori di risonanza e messa a punto di configurazioni che possano scongiurare situazioni non controllabili
+vii) Studio della fatica degli elementi interessati
+viii) Progettazione del processo produttivo
+Tale studio verrà condotto da una società specializzata nello studio di dispositivi di ammortizzazione meccanica.
+2) Realizzazione del prototipo, verrà eseguito dalla società CNC Factory specializzata nella realizzazione e produzione di pezzi meccanici.
+3) Verifica sperimentale sia di qualificazione del pezzo che di applicazione dello stesso ad una struttura appositamente realizzata su tavola vibrante.
+Lo studio verrà condotto dal laboratorio prove sui materiali dell’Università della Basilicata.
+4) La modellizzazione ed il calcolo strutturale su modelli di edifici reali in diverse configurazioni strutturali, sollecitati con differenti accellerogrammi rappresentativi di terremoti reali, con analisi dinamica non lineare, come previsto per tali dispositivi in normativa.
+Tale studio verrà condotto dalla società ASI Europa società leader specializzata nel calcolo strutturale AEM.
+5) Messa in produzione, standardizzazione del processo (inclusa la procedura di calcolo strutturale e gli studi applicativi sugli edifici reali), e commercializzazione del dispositivo.
+6) Messa in opera
+7) Manutenzione periodica dei dispositivi
+Nello specifico, scopo dello studio sarà provare che il sistema è in grado di attenuare le sollecitazioni trasmesse dal terreno agli edifici durante un evento sismico, filtrando le frequenze maggiormente dannose.
+Generalmente, tra le diverse attività sismiche, le strong motion risultano essere le più dannose sui fabbricati in quanto caratterizzate da vibrazioni con ampiezza e periodo tali da produrre danni su ambiente e infrastrutture:
+• Ampiezza: 0.001 g ÷ 1 g;
+• Frequenza: 0.06 Hz ÷ 25 Hz.
+Verrà dunque studiata la configurazione del dispositivo conducendo, successivamente, analisi statiche e dinamiche sul pezzo, per analizzarne e verificarne il comportamento.
+Nella fattispecie, dopo aver ipotizzato una configurazione preliminare del dispositivo, si verificherà la risposta dello stesso sottoposto a sollecitazioni di tipo statiche incrementate gradualmente fino al raggiungimento delle condizioni di snervamento del cavo d’acciaio. Inoltre, verranno analizzate le deformazioni indotte sull’elastomero, funzione del tipo di polimero da impiegare durante le analisi statiche e dinamiche. Le deformazioni indotte sull’elastomero dipenderanno dal tipo di polimero utilizzato, che sarà pertanto oggetto di studio uno studio simulato, i cui risultati attesi dovranno poi essere confermati dalle prove sperimentali.
+In ultimo sarà condotto uno studio degli effetti dissipativi legati alla tipologia di sistema di smorzamento/assorbimento delle sollecitazioni previste.
+Ultimata la fase di ingegnerizzazione del prototipo sarà possibile la realizzazione del dispositivo prototipale.
+Una volta costruito, il prototipo e catalogato in differenti configurazioni e tipologie, verrà montato su un modello per la prova di caratterizzazione del pezzo e per le prove su tavola vibrante, che verrà eseguita da laboratori specializzati accreditati e/o istituti di ricerca, nello specifico Università degli Studi della Basilicata, laboratorio di prove sui materiali.
+La tavola sottoporrà il provino a movimenti oscillatori, rendendo possibile l'osservazione del comportamento dinamico delle deformazioni della struttura.
+Saranno, quindi, osservabili i fenomeni legati al filtraggio delle frequenze al controllo dei periodi di oscillazione delle strutture alle curve di isteresi di dissipazione energetica del dispositivo, di effetti del secondo ordine e di fenomeni di fatica dei materiali. Saranno, inoltre, registrati i dati sperimentali che consentiranno la modellizzazione, la caratterizzazione, la catalogazione e l’implementazione seriale del dispositivo su scala industriale.
+Alla fase sperimentale seguirà la fase di calcolo in cui, il dispositivo inserito opportunamente in strutture reali, con le caratteristiche proprie, già testate nella fase sperimentale, potrà esprimere pienamente, tutte le potenzialità del sistema.
+Infine, terminata la fase di implementazione sarà possibile procedere con la progettazione produttiva.
+Determinato l’oggetto finale sarà importante studiare i progetti di assemblaggio, dall'origine fino all'inizio della produzione.
+La capacità di sfruttare i dati 3D dei prodotti e delle risorse agevolerà la validazione, l'ottimizzazione e l'allestimento virtuale del processo produttivo, riducendo i tempi di avvio e aumentando la qualità della produzione.
+Il Process Simulate permetterà di verificare la fattibilità del processo di assemblaggio, convalidando le caratteristiche di raggiungibilità, prossimità e collisioni, grazie alla simulazione globale dell'intero processo di assemblaggio del prodotto e degli strumenti necessari.
+La creazione automatica delle sequenze di assemblaggio consentirà di migliorare la produttività del processo di pianificazione. Strumenti quali sezioni, misurazioni e rilevazione delle collisioni permetteranno di verificare e ottimizzare in modo dettagliato le situazioni di assemblaggio.
+Infine, per poter procedere con l’avvio della produzione e commercializzazione sarà necessaria la vidimazione tecnico-amministrativa del sistema LE.A.D. da parte del Consiglio Superiore dei Lavori Pubblici.
+La società Mediterranea, ritiene indispensabile, la ricerca di soci finanziatori o società leader nel settore dell’adeguamento e miglioramento sismico dei fabbricati, da affiancare alla propria azione societaria, al fine di sfruttare al meglio le forti opportunità offerte dal settore.
+E’ stato condotto uno studio, sullo stato dell’arte del mercato dei dissipatori sismici.
+Sono stati individuati i principali competitor, è stata quantificata la dimensione della vulnerabilità sismica del patrimonio edificato italiano.
+Tali azioni conoscitive hanno permesso di stimare il mercato potenziale e di individuare le principali criticità per il time to market.
+In particolare, sono state analizzate le barriere all’ingresso del mercato e sono state elaborate le azioni necessarie per superarle.
+Altresì, data la natura di un mercato fortemente orientato alla ricerca e sviluppo di soluzioni innovative, si ritiene che il fattore tempo giochi un ruolo determinante per il successo del prodotto sul mercato.
+Mediterrranea S.r.L.s. Viale dei Pentri 117/a 86170 Isernia (IS)
+Viale dei Pentri 117/a 86170 Isernia tel/fax 0865 299759 – p.iva 00977110949
+studio.mediterrranea@gmail.com www.mediterrenea-lide.com
+V/1-2020</t>
+        </is>
+      </c>
+      <c r="BH2" t="inlineStr">
+        <is>
+          <t>The particularity of the invention consists precisely in the adoption of the aforementioned joints, called anti-seismic joints with elastomers (indicated by the acronym "GAE").
+This joint is highly standardized to allow its assembly in extremely short times, in a great variety of geometric configurations of the load bearing structures of a building.
+The GAE is made up of a specially designed cylindrical joint which houses the stringing head of a threaded rod tie rod. The adoption of threaded rods allows to minimize the overall dimensions of the clamping system and allows, by simply screwing a nut, to give a pretensioning of the tie rod, which will be calibrated using torque wrenches. The tie head housing system provides for the interposition of a Newton-type elastomeric element with an elasto-plastic characterization, which gives it the ability to dissipate energy.
+By dosing the pre-tensioning of the tie rod and the elastic response of the elastomer cartridge housed in the joint, it is possible to "modulate" the reaction of the tie rod and "pilot" the response in seismic conditions of the entire load-bearing structure of the building.
+In summary, the characteristics of the GAE are:
+1. Dissipative capacity modifiable according to needs;
+2. Ease of assembly
+3. Easy and inexpensive restoration following an earthquake and periodic maintenance, thanks to the replacement of the elastomeric element only housed in the joint (cartridge);
+4. Limited dimensions and weight for easy transport and assembly;
+5. Reduced assembly times.
+For the exploitation of patent technology, analytical studies must be undertaken in order to validate and pursue system improvements; the compulsory stages of the prototype development necessary for the validation of the system by the Superior Council of Public Works have been identified.
+The company is the beneficiary of the loan of Euro 131,742.88 obtained through the European PATENT + loan granted by INVITALIA, a national company for the attraction of investments and the development of a SPA company.
+The key step of the procedural process will be the creation of an experimental prototype, tested on a vibrating table and analyzed in order to proceed with modeling.
+Therefore, the services necessary for the development and subsequent validation of the system are:
+1) Analysis and industrialization of the device, which includes:
+a) Study, design and engineering of the prototype:
+i) Modeling and engineering;
+ii) Static and dynamic modeling analysis on the device;
+iii) Dissipative effects analysis;
+iv) Frequency filtering analysis
+v) Analysis of the hysteresis curves and the dissipative capacity of the device
+vi) Analysis of the resonance factors and development of configurations that can avoid situations that cannot be controlled
+vii) Study of the fatigue of the elements involved
+viii) Design of the production process
+This study will be conducted by a company specializing in the study of mechanical cushioning devices.
+2) Realization of the prototype, will be carried out by the CNC Factory company specialized in the realization and production of mechanical parts.
+3) Experimental verification of both the qualification of the piece and its application to a structure specially made on a vibrating table.
+The study will be conducted by the materials testing laboratory of the University of Basilicata.
+4) Modeling and structural calculation on models of real buildings in different structural configurations, stressed with different accelerograms representative of real earthquakes, with non-linear dynamic analysis, as required for such devices in the legislation.
+This study will be conducted by ASI Europa, a leading company specializing in AEM structural calculation.
+5) Production, standardization of the process (including the structural calculation procedure and application studies on real buildings), and marketing of the device.
+6) Implementation
+7) Periodic maintenance of the devices
+Specifically, the purpose of the study will be to prove that the system is able to attenuate the stresses transmitted from the ground to buildings during a seismic event, filtering the most damaging frequencies.
+Generally, among the various seismic activities, strong motion are the most harmful on buildings as they are characterized by vibrations with amplitude and period such as to produce damage to the environment and infrastructure:
+• Amplitude: 0.001 g ÷ 1 g;
+• Frequency: 0.06 Hz ÷ 25 Hz.
+The configuration of the device will therefore be studied, subsequently carrying out static and dynamic analyzes on the piece, to analyze and verify its behavior.
+In this case, after having assumed a preliminary configuration of the device, the response of the device will be verified subjected to static stresses gradually increased until the yield conditions of the steel cable are reached. Furthermore, the deformations induced on the elastomer will be analyzed, depending on the type of polymer to be used during the static and dynamic analyzes. The deformations induced on the elastomer will depend on the type of polymer used, which will therefore be the subject of a simulated study, the expected results of which must then be confirmed by experimental tests.
+Finally, a study of the dissipative effects related to the type of damping / absorption system of the foreseen stresses will be carried out.
+Once the prototype engineering phase has been completed, it will be possible to create the prototype device.
+Once built, the prototype and cataloged in different configurations and types, will be mounted on a model for the characterization test of the piece and for the vibrating table tests, which will be performed by accredited specialized laboratories and / or research institutes, specifically University of Basilicata, materials testing laboratory.
+The table will subject the specimen to oscillatory movements, making it possible to observe the dynamic behavior of the deformations of the structure.
+Therefore, the phenomena related to the filtering of frequencies to the control of the periods of oscillation of the structures to the hysteresis curves of energy dissipation of the device, of second order effects and of material fatigue phenomena, will be observable. The experimental data will also be recorded that will allow the modeling, characterization, cataloging and serial implementation of the device on an industrial scale.
+The experimental phase will be followed by the calculation phase in which the device properly inserted in real structures, with its own characteristics, already tested in the experimental phase, will be able to fully express all the potential of the system.
+Finally, once the implementation phase is complete, it will be possible to proceed with the production design.
+Once the final object has been determined, it will be important to study the assembly projects, from the origin to the start of production.
+The ability to leverage 3D product and asset data will facilitate the validation, optimization and virtual setup of the production process, reducing start-up times and increasing production quality.
+The Process Simulate will allow to verify the feasibility of the assembly process, validating the characteristics of reachability, proximity and collisions, thanks to the global simulation of the entire assembly process of the product and the necessary tools.
+Automatic creation of assembly sequences will improve the productivity of the planning process. Tools such as sections, measurements and collision detection will allow you to check and optimize assembly situations in detail.
+Finally, in order to proceed with the start of production and marketing, the technical-administrative endorsement of the LE.A.D. system will be required. by the Higher Council of Public Works.
+The Mediterranea company considers it essential to find financing partners or leading companies in the sector of seismic adaptation and improvement of buildings, to complement its corporate action, in order to make the most of the strong opportunities offered by the sector.
+A study was conducted on the state of the art of the seismic dissipator market.
+The main competitors were identified, the size of the seismic vulnerability of the Italian built heritage was quantified.
+These cognitive actions made it possible to estimate the potential market and to identify the main critical issues for the time to market.
+In particular, the barriers to market entry were analyzed and the necessary actions were developed to overcome them.
+Furthermore, given the nature of a market strongly oriented towards the research and development of innovative solutions, it is believed that the time factor plays a decisive role in the success of the product on the market.
+Mediterrranea S.r.L.s. Viale dei Pentri 117 / a 86170 Isernia (IS)
+Viale dei Pentri 117 / a 86170 Isernia tel / fax 0865 299759 - VAT number 00977110949
+studio.mediterrranea@gmail.com www.mediterrenea-lide.com
+V / 1-2020</t>
+        </is>
+      </c>
+      <c r="BI2" t="inlineStr">
+        <is>
+          <t>Lo stock immobiliare italiano si compone di oltre 29 milioni di abitazioni per 60 milioni di residenti; di queste, 10 milioni circa sono costruite nelle zone sismiche più a rischio: 1,4 milioni sono ubicate nella zona 1 e circa 9 milioni in zona 2. Sono invece 8,5 milioni le abitazioni collocate in zona 3 e 9,4 milioni, infine, in zona 4. Inoltre, il patrimonio edilizio residenziale italiano tende al vecchio. Il capitale edilizio e quello infrastrutturale del Paese sono entrati in un ciclo di obsolescenza crescente. Dei 12,2 milioni di edifici residenziali censiti dall’Istat, per esempio, 7,2 milioni (il 60%) sono stati costruito prima del 1980; 5,2 milioni (42,5%) hanno più di 50 anni. Più della metà delle abitazioni - oltre 16 milioni - sono state realizzate prima del 1970.
+Almeno un terzo degli immobili andrebbe adeguato.
+Secondo le stime del Consiglio Nazionale degli Ingegneri servirebbero un po’ più di 90 miliardi di euro per mettere in sicurezza il patrimonio residenziale italiano; per la Protezione Civile ne potrebbero addirittura bastare poco più di 50.
+Quindi possiamo stimare in 70 miliardi di euro (dato medio delle due stime sopracitate) il mercato totale disponibile (TAM).
+Per la stima del mercato raggiungibile (SAM) bisogna tener conto della percezione del rischio sismico da parte degli italiani. Dall’analisi del comportamento degli italiani risulta che tale rischio è sottostimato.
+Prova ne è l’incidenza delle ristrutturazioni antisismiche sul totale delle ristrutturazioni effettuate dagli italiani nel biennio 2015-2016: gli immobili per i quali sono stati dichiarati interventi antisismici sono poco più di 33.000, mentre gli immobili per i quali sono stati dichiarati lavori di ristrutturazione, solo nell’anno 2016, sono quasi 1,5 milioni.
+Nel periodo 2013-2016 sono stati effettuati poco più di 195 mila interventi antisismici. L’ammontare totale di spesa per questa categoria di opere è stato pari a oltre 872 milioni di euro.
+Per il 2020, l'A.N.C.E. prevede un incremento dell'1,5% per investimenti in manutenzione straordinaria dello stock abitativo. La stima tiene conto, tra l'altro, dell’impatto sui livelli produttivi degli interventi finalizzati alla riduzione del rischio sismico legati al sisma bonus.
+Quindi, possiamo calcolare il SAM di riferimento come prodotto fra la spesa media per intervento ed il numero di interventi annui aumentato dell'1,5%, cioè poco meno di 74,9 milioni di euro.
+Tali studi sono precedenti all’emergenza sanitaria dovuta al COVID 19.
+Per la determinazione del SOM (mercato realmente ottenibile) è stato necessario tener conto del grado di concentrazione del mercato e del vantaggio competitivo che si pensa di poter ottenere con il sistema LE.A.D.
+Le tecniche più innovative, e più vicine al sistema proposto, attualmente disponibili sul mercato, si basano sull’utilizzo di dissipatori isteretici tipo Brad (Buckling Restrained Axial Damper).
+Tale tecnica prevede, generalmente, il diretto inserimento dei dispositivi all’interno della maglia strutturale, tali dispositivi hanno dimensioni considerevoli ma avendo un funzionamento che prevede sia la trazione che la compressione, per motivi di instabilità e di ingombro, possono raggiungere solo luci limitate.
+La particolarità del sistema LE.A.D, consiste nell'adozione di tiranti ad alto limite elastico, che permettono un contenimento delle dimensioni delle controventature, agendo solo in trazione, non avendo quindi problematiche di instabilità, tanto da poter essere installato e movimentato in cantiere da poche persone senza l’ausilio di attrezzature speciali, il peso dell’apparecchio infatti non supera i 25 Kg, a vantaggio anche degli aspetti estetico-funzionali, in quanto il sistema è facilmente occultabile, oltre che ad una estrema semplicità e rapidità di messa in opera, con riduzione sostanziale sia dei tempi di esecuzione delle lavorazioni, che dell’impatto e dell’invasività delle stesse sulla struttura esistente e sulle rifiniture del fabbricato su cui si interviene.
+Inoltre il sistema di incatenamento, che può essere considerato una estensione del sistema tradizionale catena-capochiave, permette di intervenire su luci molto più estese rispetto al sistema BRAD, essendo basato esclusivamente sulla trazione e sulla legatura, meccanismo che è scevro dai problemi di svergolamento per instabilità dovuta a carico di punta.
+Tale vantaggio è quantificabile in un minor costo per l’utente, oltre che una maggiore flessibilità di messa in opera e una minore invasività sull’esistente.
+Nella corrente pratica di miglioramento sismico, circa l’85% dei costi è determinato dagli interventi accessori di ripristino delle rifiniture ed impianti, costi che vengono notevolmente ridotti dall’applicazione del sistema LE.A.D., in quanto la cucitura delle strutture non richiede interventi invasivi sull’edificio e gran parte delle rifiniture e degli impianti può essere preservato.
+Il vantaggio tecnologico e funzionale del sistema LE.A.D. consentirà all’azienda di superare le barriere tecnologiche all’entrata del mercato di riferimento, poiché il sistema è fortemente innovativo rispetto ai sistemi già presenti sul mercato.
+Tenuto conto della posizione di vantaggio che si presume di poter assumere rispetto ai competitor, possiamo procedere ad una stima (prudenziale) del SOM di riferimento.
+Per il primo anno si prevede di poter raggiungere almeno il 2% del SAM, corrispondente ad un fatturato di poco al di sotto di 1,5 milioni di euro.
+Tale previsione andrà ad aumentare negli anni successivi, e sarà proporzionale alla capacità di penetrazione sul mercato, date le condizioni ed il vantaggio competitivo del sistema, è ragionevole ipotizzare un incremento prudenziale del 10% annuo.
+Si presume pertanto che a fine vita del brevetto, senza ipotizzare scenari più favorevoli e ulteriori sviluppi applicativi, nonché la conquista di nuovi mercati anche internazionali, l’azienda possa cumulare un montante di fatturato pari a circa 86.000.000 di euro derivanti esclusivamente dalla vendita del sistema.
+Mediterrranea S.r.L.s. Viale dei Pentri 117/a 86170 Isernia (IS)
+Viale dei Pentri 117/a 86170 Isernia tel/fax 0865 299759 – p.iva 00977110949
+studio.mediterrranea@gmail.com www.mediterrenea-lide.com
+V/1-2020</t>
+        </is>
+      </c>
+      <c r="BJ2" t="inlineStr">
+        <is>
+          <t>Attualmente non risultano sistemi concorrenti sul mercato.</t>
+        </is>
+      </c>
+      <c r="BK2" t="inlineStr">
+        <is>
+          <t>Il brevetto ci consente di adeguare in modo semplice ed innovativo ogni edificio in CA</t>
+        </is>
+      </c>
+      <c r="BL2" t="inlineStr">
         <is>
           <t>SÌ</t>
         </is>
       </c>
-      <c r="AI2" t="inlineStr">
+      <c r="BM2" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="AJ2" t="inlineStr">
+      <c r="BN2" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="AK2" t="inlineStr">
+      <c r="BO2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="BP2" t="inlineStr">
         <is>
           <t>NON RILEVATO</t>
         </is>
       </c>
-      <c r="AL2" t="inlineStr">
+      <c r="BQ2" t="inlineStr">
         <is>
           <t>NON RILEVATO</t>
         </is>
       </c>
-      <c r="AM2" t="inlineStr">
-        <is>
-          <t>InfoCert Qualified Electronic Signature CA 3</t>
-        </is>
-      </c>
-      <c r="AN2" t="inlineStr">
-        <is>
-          <t>01038800148-20251014171044</t>
-        </is>
-      </c>
-      <c r="AO2" t="inlineStr">
-        <is>
-          <t>https://i.ibb.co/zTv2Mhd2/40b03b928e72.jpg</t>
-        </is>
-      </c>
-      <c r="AP2" t="inlineStr">
-        <is>
-          <t>Disponibile (Caricato su ImgBB)</t>
-        </is>
-      </c>
-      <c r="AQ2" t="inlineStr">
+      <c r="BR2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="BS2" t="inlineStr">
+        <is>
+          <t>SÌ</t>
+        </is>
+      </c>
+      <c r="BT2" t="inlineStr">
+        <is>
+          <t>SÌ</t>
+        </is>
+      </c>
+      <c r="BU2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="BV2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="BW2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="BX2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="BY2" t="inlineStr">
         <is>
           <t>NON RILEVATO</t>
         </is>
       </c>
-      <c r="AR2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/wide-vr/</t>
-        </is>
-      </c>
-      <c r="AS2" t="inlineStr">
-        <is>
-          <t>Facebook.com/widemilan</t>
-        </is>
-      </c>
-      <c r="AT2" t="inlineStr">
+      <c r="BZ2" t="inlineStr">
         <is>
           <t>NON RILEVATO</t>
         </is>
       </c>
-      <c r="AU2" t="inlineStr">
-        <is>
-          <t>NON RILEVATO</t>
-        </is>
-      </c>
-      <c r="AV2" t="inlineStr">
-        <is>
-          <t>NON RILEVATO</t>
-        </is>
-      </c>
-      <c r="AW2" t="inlineStr">
-        <is>
-          <t>NON RILEVATO</t>
-        </is>
-      </c>
-      <c r="AX2" t="inlineStr">
-        <is>
-          <t>NON RILEVATO</t>
-        </is>
-      </c>
-      <c r="AY2" t="inlineStr">
-        <is>
-          <t>S3</t>
-        </is>
-      </c>
-      <c r="AZ2" t="inlineStr">
-        <is>
-          <t>Sul mercato</t>
-        </is>
-      </c>
-      <c r="BA2" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="BB2" t="inlineStr">
-        <is>
-          <t>Pronto</t>
-        </is>
-      </c>
-      <c r="BC2" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="BD2" t="inlineStr">
-        <is>
-          <t>Completo</t>
-        </is>
-      </c>
-      <c r="BE2" t="inlineStr">
-        <is>
-          <t>Wide VR è una startup specializzata in soluzioni 3D cutting-edge. Abbiamo realizzato diversi progetti per clienti internazionali tra cui Nike, Mapei e Italtherm. Wide VR presenta Vshop, la prima piattaforma ad abbonamento per la creazione automatizzata di shop virtuali in qualità fotorealistica compatibili con qualunque piattaforma e-commerce. Vshop risolve il problema delle scarse conversioni in ambito e-commerce dovute ad un'esperienza del prodotto limitata dall'uso della fotografia. È possibile creare shop virtuali a partire da template pensati per diverse nicchie di mercato tra cui moda, accessori e design. La navigazione degli spazi avviene via web con una qualità vicina al realismo, grazie ad un software proprietario basato su una pipeline innovativa, che combina nuove tecnologie tra cui la conversione 3D high poly e L'AI. Il modello di business ad abbonamento prevede piani economici che rendono la soluzione scalabile.</t>
-        </is>
-      </c>
-      <c r="BF2" t="inlineStr">
-        <is>
-          <t>Wide VR is specialized in cutting-edge 3D solutions. We have developed several projects for international clients including Nike, Mapei and Italtherm. Wide VR presents Vshop, the first subscription-based platform for the automated creation of photorealistic quality virtual shops compatible with any e-commerce platform. Vshop solves the problem of low conversions in e-commerce due to a product experience limited by the use of photography. Virtual shops can be created from templates designed for different market niches including fashion, accessories and design. Spaces are navigated via the web with a quality close to realism, thanks to proprietary software based on an innovative pipeline, which combines new technologies including high poly 3D conversion and AI. The subscription-based business model provides economic plans that make the solution scalable.</t>
-        </is>
-      </c>
-      <c r="BG2" t="inlineStr">
-        <is>
-          <t>Vshop è la prima piattaforma ad abbonamento per la creazione automatizzata di shop virtuali in qualità fotorealistica compatibili con qualunque piattaforma e-commerce. Vshop risolve il problema delle scarse conversioni in ambito e-commerce dovute ad un'esperienza del prodotto limitata dall'uso della fotografia. È possibile creare shop virtuali a partire da template pensati per diverse nicchie di mercato tra cui moda, accessori e design. La navigazione degli spazi avviene via web con una qualità vicina al realismo, grazie ad un software proprietario basato su una pipeline innovativa, che combina nuove tecnologie tra cui la conversione 3D high poly e L'AI. Il modello di business ad abbonamento prevede piani economici che rendono la soluzione scalabile.</t>
-        </is>
-      </c>
-      <c r="BH2" t="inlineStr">
-        <is>
-          <t>Vshop is the first subscription-based platform for the automated creation of photorealistic quality virtual shops compatible with any e-commerce platform. Vshop solves the problem of low conversions in e-commerce due to a product experience limited by the use of photography. Virtual shops can be created from templates designed for different market niches including fashion, accessories and design. Spaces are navigated via the web with a quality close to realism, thanks to proprietary software based on an innovative pipeline, which combines new technologies including high poly 3D conversion and AI. The subscription-based business model provides economic plans that make the solution scalable.</t>
-        </is>
-      </c>
-      <c r="BI2" t="inlineStr">
-        <is>
-          <t>Saas con abbonamento mensile</t>
-        </is>
-      </c>
-      <c r="BJ2" t="inlineStr">
-        <is>
-          <t>In Italia i competitor usano tecnologie poco avanzate come i video 360, noi lavoriamo sui vari verticali in real-time 3D con pipeline specifiche.</t>
-        </is>
-      </c>
-      <c r="BK2" t="inlineStr">
-        <is>
-          <t>Real-time 3D with photorealistic output, fully integrated with AI.</t>
-        </is>
-      </c>
-      <c r="BL2" t="inlineStr">
+      <c r="CA2" t="inlineStr">
         <is>
           <t>SÌ</t>
         </is>
       </c>
-      <c r="BM2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="BN2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="BO2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="BP2" t="inlineStr">
-        <is>
-          <t>EMILIA-ROMAGNA, LOMBARDIA, TOSCANA</t>
-        </is>
-      </c>
-      <c r="BQ2" t="inlineStr">
-        <is>
-          <t>Unione europea, America settentrionale</t>
-        </is>
-      </c>
-      <c r="BR2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="BS2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="BT2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="BU2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="BV2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="BW2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="BX2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="BY2" t="inlineStr">
-        <is>
-          <t>NON RILEVATO</t>
-        </is>
-      </c>
-      <c r="BZ2" t="inlineStr">
-        <is>
-          <t>NON RILEVATO</t>
-        </is>
-      </c>
-      <c r="CA2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
       <c r="CB2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÌ</t>
         </is>
       </c>
       <c r="CC2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="CD2" t="n">
         <v>0</v>
@@ -1335,44 +1514,229 @@
         </is>
       </c>
       <c r="CK2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="CL2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CM2" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="CN2" t="inlineStr">
         <is>
-          <t>Team composto da CEO e COO con laurea triennale, co-founder, solido</t>
+          <t>Team composto da 3 fondatori con laurea magistrale e un dottorato, ruoli C-Level completi</t>
         </is>
       </c>
       <c r="CO2" t="inlineStr">
         <is>
-          <t>WIDE VR SVOLGE ATTIVITA' DI SVILUPPO DI SOFTWARE, PIATTAFORME DIGITALI, SERVIZI DIGITALI, APP E CONTENUTI MULTIMEDIALI NELL'AMBITO DELLE APPLICAZIONI DI TECNOLOGIE 3D, REALTA' VIRTUALE E PER IL METAVERSO. LA SOCIETA' SVOLGE INOLTRE ATTIVITA' DI RICERCA, SVILUPPO E INNOVAZIONE NEL CAMPO DELLE TECNOLOGIE DIGITALI APPLICATE ALL'E-COMMERCE E IN AMBITO DI PROGRAMMAZIONE, SVILUPPO DI PROGETTI E LA FORNITURA DI SERVIZI LEGATI ALLA TECNOLOGIA BLOCKCHAIN. --------------------------------------------------- SPESE IN RICERCA E SVILUPPO PER L'ESERCIZIO 2023 PARI A EURO 90.199,26 A FRONTE DI UN TOTALE DEL VALORE DELLA PRODUZIONE PARI A EURO 70.455,00</t>
+          <t>LA SOCIETA' SI PROPONE DI METTERE IN PRODUZIONE E COMMERCIALIZZARE UN DISPOSITIVO ANTISISMICO INNOVATIVO DI CUI LA STESSA SOCIETA' E' LICENZIATARI. LE SPESE DI RICERCA E SVILUPPO RICUARDANO TRE FASI 1) INDUSTRAILIZZAZIONE DEL DISPOSITIVO 2) MODELLI DI CALCOLO STRUTTURALI PER VALUTARE LA RISPOSTA DEL DISPOSITIVO AD AZIONI SISMICHE ELABORATE SIA SULLO STESSO COMPONENTE IN TERMINI DI TENSIONI 1) INDUSTRAILIZZAZIONE DEL DISPOSITIVO 2) MODELLI DI CALCOLO STRUTTURALI PER VALUTARE LA RISPOSTA DEL DISPOSITIVO AD AZIONI SISMICHE ELABORATE SIA SULLO STESSO COMPONENTE CHE RIFERITI ALL'INTERAZIONE DISPOSITIVO ORGANISMO STRUTTURALE. LE ANALISI SONO DI TIPO DINAMICO NON LINEARE. 3)CAMPAGNA SPERIMENTALE CONDOTTA DA UN'ENTE ACCREDITATO. LA SOCIETA' MEDITERRENEA SRLS, LICENZIATARIA DI BREVETTO PER INVENZIONE INDUSTRIALE LE.A.D., HA INIZIATO L'ATTIVITA' IN DATA 16/01/2020. L'OGGETTO SOCIALE CONSISTE IN LAVORAZIONI SPECIALIZZATE SU COSTRUZIONE IN CEMENTO ARMATO. NELLO SPECIFICO, L'OGGETTO DI DOMANDA DI FINANZIAMENTO ATTIENE AD UN SISTEMA STRUTTURALE DI CONTROVENTATURA DI STRUTTURE INTELAIATE IN ACCIAIO/CLS ARMATO (LE.A.D.), OVVERO DI SETTI MURARI PORTANTI, CHE PERMETTE DI MODIFICARE LA RISPOSTA DELL'ORGANISMO STRUTTURALE IN CASO DI SISMA. TUTTO IL SISTEMA E' IMPERNIATO SULLA REALIZZAZIONE DI CONTROVENTI "DISSIPATIVI" COSTITUITI DA TIRANTI COLLEGATI ALLA RESTANTE STRUTTURA ATTRAVERSO PARTICOLARI GIUNTI CHE HANNO CAPACITA' DI DISSIPARE ENERGIA GRAZIE AD ELEMENTI IN ELASTOMERO. LA PARTICOLARITA' DELL'INVENZIONE CONSISTE PROPRIO NELLA ADOZIONE DEI PREDETTI GIUNTI, DEFINITI "GIUNTI ANTISISMICI ELASTOMERICI" (GAE), AD ELEVATA STANDARDIZZAZIONE PER CONSENTIRNE IL MONTAGGIO, IN TEMPI ESTREMAMENTE RAPIDI, IN UNA GRANDE VARIETA' DI CONFIGURAZIONI GEOMETRICHE DELLE STRUTTURE PORTANTI DI UN EDIFICIO. ESSI SONO PROGETTATI, AL MOMENTO, IN DUE DIVERSE VERSIONI PER CONSENTIRNE SIA L'UTILIZZO ALL'INTERNO DI STRUTTURE INTELAIATE SIA PER INSTALLAZIONE A RIDOSSO DI SETTI MURARI. IL SISTEMA DI LEGATURE ANTISISMICHE DISSIPATIVE SI BASA SULLA REALIZZAZIONE DI LEGATURE A CONTROVENTI "DISSIPATIVI" COSTITUITI DA TIRANTI COLLEGATI ALLA STRUTTURA ATTRAVERSO PARTICOLARI GIUNTI CHE HANNO LA CAPACITA' DI DISSIPARE ENERGIA GRAZIE AD ELEMENTI IN ELASTOMERO. LA PARTICOLARITA' DELL'INVENZIONE CONSISTE PROPRIO NELL'ADOZIONE DEI PREDETTI GIUNTI, DENOMINATI GIUNTI ANTISISMICI CON ELASTOMERI (INDICATO DALL'ACRONIMO "GAE"). TALE GIUNTO PRESENTA ELEVATA STANDARDIZZAZIONE PER CONSENTIRNE IL MONTAGGIO IN TEMPI ESTREMAMENTE RAPIDI, IN UNA GRANDE VARIETA' DI CONFIGURAZIONI GEOMETRICHE DELLE STRUTTURE PORTANTI DI UN EDIFICIO. IL GAE E' COSTITUITO DA UNO SNODO CILINDRICO, APPOSITAMENTE CONCEPITO, CHE OSPITA LA TESTA DI TESATURA DI UN TIRANTE IN BARRA FILETTATA. L'ADOZIONE DI BARRE FILETTATE PERMETTE DI CONTENERE AL MINIMO L'INGOMBRO DEL SISTEMA DI SERRAGGIO E PERMETTE, TRAMITE IL SEMPLICE AVVITAMENTO DI UN DADO, DI CONFERIRE UN PRETENSIONAMENTO DEL TIRANTE, CHE VERRA' CALIBRATO TRAMITE CHIAVI DINAMOMETRICHE. IL SISTEMA DI ALLOGGIAMENTO DELLA TESTA TIRANTE PREVEDE L'INTERPOSIZIONE DI UN ELEMENTO ELASTOMERICO DI TIPO NEWTON A CARATTERIZZAZIONE ELASTO-PLASTICA, CHE CONFERISCE LA CAPACITA' DI DISSIPARE ENERGIA. ANDANDO A DOSARE IL PRETENSIONAMENTO DEL TIRANTE E LA RISPOSTA ELASTICA DELLA CARTUCCIA DI ELASTOMERO ALLOGGIATA NEL GIUNTO SI RIESCE A "MODULARE" LA REAZIONE DEL TIRANTE ED A "PILOTARE" LA RISPOSTA IN CONDIZIONI SISMICHE DELL'INTERA STRUTTURA PORTANTE DELL'EDIFICIO. IN SINTESI LE CARATTERISTICHE DEL GAE SONO: 1. CAPACITA' DISSIPATIVA MODIFICABILE IN FUNZIONE DELLE NECESSITA'; 2. FACILITA' DI MONTAGGIO 3. FACILITA' ED ECONOMICITA' DI RIPRISTINO A SEGUITO DI SISMA E DI MANUTENZIONE PERIODICA, GRAZIE ALLA SOSTITUIBILITA' DEL SOLO ELEMENTO ELASTOMERICO ALLOGGIATO NEL GIUNTO (CARTUCCIA); 4. DIMENSIONI E PESO CONTENUTI PER UN AGEVOLE TRASPORTO E MONTAGGIO; 5. RIDOTTI TEMPI DI MONTAGGIO.</t>
         </is>
       </c>
       <c r="CP2" t="inlineStr">
         <is>
-          <t>TITOLI ED ESPERIENZE PROFESSIONALI NON DICHIARATI COME REQUISITO DELLA STARTUP</t>
+          <t>LA MEDITERRANEA SRLS AVRA' COME SCOPO LO SVILUPPO, LA PRODUZIONE E LA COMMERCIALIZZAZIONE DEL DISPOSITIVO LE.A.D. I SOCI DELLA SUDDETTA SOCIETA' SONO: ARCH. PIER LUIGI PACITTI, ING. NICOLETTA BUCCI, ING. SILVIA BUCCI. L'ARCH. PACITTI HA MATURATO UNA PROFONDA ESPERIENZA NEL CAMPO TECNICO, CON PARTICOLARE RIGUARDO PER I METODI DI CATALOGAZIONE E RILIEVO DI DETRATTORI AMBIENTALI E DI VERIFICA DI STRUMENTI URBANISTICI. SI EVIDENZIA, NELLO SPECIFICO, L'ULTRAVENTENNALE ESPERIENZA ACQUISITA NEL CAMPO PROCEDURALE CON PARTICOLARE RIGUARDO PER QUEL CHE RIGUARDA L'ITER BUROCRATICO-AMMINISTRATIVO DELLE PRATICHE PROGETTUALI, DALLE AUTORIZZAZIONI, ALLE LEGGI AMBIENTALI, URBANISTICHE, SUL RISPARMIO ENERGETICO, ANTISISMICHE, TECNOLOGICHE ED ELETTRICHE. L'ING. NICOLETTA BUCCI, DOPO LA LAUREA IN INGEGNERIA CHIMICA, HA MATURATO PROFONDA CONOSCENZA IN IMPIANTISTICA CHIMICA PRESSO LA MULTINAZIONALE SAIPEM DI MILANO. L'ING. SILVIA BUCCI, LAUREATASI PRESSO LA FACOLTA' DI INGEGNERIA DELL'INFORMAZIONE, INFORMATICA E STATISTICA DELLA SAPIENZA DI ROMA, E' ATTUALMENTE IMPEGNATA IN UN DOTTORATO DI RICERCA PRESSO IL POLITECNICO DI TORINO DAL TITOLO DOMAIN GENERALIZATION VIA SELF-SUPERVISED LEARNING. IL SOCIO PACITTI, DATA L'ESPERIENZA, SI OCCUPERA' DELLA PARTE BUROCRATICA E COORDINERA' IL LAVORO DEGLI ALTRI DUE SOCI. IL SOCIO NICOLETTA BUCCI SI OCCUPERA' DELLO SVILUPPO E DELL'ANALISI DEI MATERIALI. IL SOCIO SILVIA BUCCI SI OCCUPERA' DELL'ANALISI E DELL'ELABORAZIONE DEI DATI. IN UN'OTTICA DI CONTENIMENTO DEI COSTI FISSI IN FASE DI AVVIO DELL'AZIENDA, RISULTA INOPPORTUNO PROCEDERE AD UNA PRODUZIONE DIRETTA DEL DISPOSITIVO. QUINDI, IN UNA PRIMA FASE, L'AZIENDA RITIENE OPPORTUNO ESTERNALIZZARE LA PRODUZIONE. ANCHE PER LA PROMOZIONE E LA COMMERCIALIZZAZIONE DEL DISPOSITIVO L'AZIENDA SI AVVARRA' DI FIGURE ESTERNE.</t>
         </is>
       </c>
       <c r="CQ2" t="inlineStr">
         <is>
-          <t>LA STARTUP E' INCUBATA PRESSO L'INCUBATORE E ACCELERATORE STARTUPIACENZA - URBAN HUB PIACENZA</t>
+          <t>AI FINI DELLA VALIDAZIONE INGEGNERISTICA DEL BREVETTO IL SISTEMA DEVE ESSERE IN GRADO DI FILTRARE LE FREQUENZE E LE AMPIEZZE PIU' GRAVOSE PER L'EDIFICIO TRASMESSE DAL TERRENO, ATTENUANDONE I PICCHI, CON EFFETTI DISSIPATIVI DELLE ENERGIE ATTIVATE. LE ATTIVITA' SISMICHE CHE HANNO EFFETTI DANNOSI SUI FABBRICATI SONO LE ATTIVITA' STRONG MOTION, CARATTERIZZATE DA VIBRAZIONI IN AMPIEZZA E PERIODO TALI DA PRODURRE DANNI SU AMBIENTE E INFRASTRUTTURE, SI TRATTA DI VIBRAZIONI DI AMPIEZZE COMPRESE TRA 0.001 G E 1 G CON FREQUENZE COMPRESE TRA 0.06 HZ E 25 HZ. NON SI E' ANCORA IN GRADO AL MOMENTO DI PREFIGURARE UNA CONFORMAZIONE STANDARD DELL'APPARECCHIO, CHE DEVE ESSERE APPUNTO OGGETTO DI STUDIO. QUINDI, I SERVIZI NECESSARI ALLO SVILUPPO E ALLA SUCCESSIVA VALIDAZIONE DEL SISTEMA SONO: 1 ANALISI E INDUSTRIALIZZAZIONE DELL'APPARECCHIO DA PARTE DELLA MO.S.A.I.C. S.R.L., CHE INCLUDE: A) STUDIO, PROGETTAZIONE ED INGEGNERIZZAZIONE DEL PROTOTIPO: I) MODELLAZIONE E INGEGNERIZZAZIONE; II) ANALISI STATICHE E DINAMICHE MODELLISTICHE SUL DISPOSITIVO; III) ANALISI EFFETTI DISSIPATIVI; IV) ANALISI DEL FILTRAGGIO DELLE FREQUENZE V) ANALISI DELLE CURVE DI ISTERESI E DELLA CAPACITA' DISSIPATIVA DELL'APPARECCHIO VI) ANALISI DEI FATTORI DI RISONANZA E MESSA A PUNTO DI CONFIGURAZIONI CHE POSSANO SCONGIURARE SITUAZIONI NON CONTROLLABILI VII) STUDIO DELLA FATICA DEGLI ELEMENTI INTERESSATI 2 REALIZZAZIONE DEL PROTOTIPO: IL PROTOTIPO VERRA' REALIZZATO DALLA DITTA CNC FACTORY S.R.L.S., SPECIALIZZATA NELLA REALIZZAZIONE DI PEZZI SPECIALI IN ACCIAIO. 3) VERIFICA SPERIMENTALE SIA DI QUALIFICAZIONE DEL PEZZO CHE DI APPLICAZIONE DELLO STESSO AD UNA STRUTTURA APPOSITAMENTE REALIZZATA SU TAVOLA VIBRANTE, SI OCCUPERA' DELLO STUDIO DI TALI ASPETTI SPERIMENTALI IL LABORATORIO PROVE SU MATERIALI E STRUTTURE DELL' UNIVERSITA' DELLA BASILICATA, STRUTTURA DI ECCELLENZA NEL CAMPO DELLE COSTRUZIONI. 4 LA MODELLIZZAZIONE ED IL CALCOLO STRUTTURALE SU MODELLI DI EDIFICI REALI IN DIVERSE CONFIGURAZIONI STRUTTURALI, SOLLECITATI CON DIFFERENTI ACCELLEROGRAMMI RAPPRESENTATIVI DI TERREMOTI REALI, CON ANALISI DINAMICA NON LINEARE, COME PREVISTO PER TALI DISPOSITIVI IN NORMATIVA, SARA' ESEGUITA DALLA DITTA ASI TRA I LEADER MONDIALI NEL CAMPO DELL'ANALISI STRUTTURALE, DETENTRICE DEL SOFTWARE EXTREME LOADING, CHE LAVORA IN CODICE AEM (APPLIED ELEMENT METHOD) UN METODO DECISAMENTE PIU' AVANZATO, AFFIDABILE E POTENTE DEI NORMALI METODI IN USO NEI PROGRAMMI DI CALCOLO BASATI SUL METODO FEM (FINITE ELEMENT METHOD). 5 PROGETTAZIONE DEL PROCESSO PRODUTTIVO DA PARTE DELLA MO.S.A.I.C. S.R.L IL SERVIZIO DELLA MO.S.A.I.C. S.R.L. CONSISTE IN UNO STUDIO CHE PERMETTA DI VALIDARE VIRTUALMENTE IL GIUNTO ANTISISMICO GAE ATTRAVERSO OPPORTUNE MODELLAZIONI CONDOTTE CON SOFTWARE SPECIFICI DI SETTORE. NELLO SPECIFICO, SCOPO DELLO STUDIO SARA' PROVARE SE IL SISTEMA E' IN GRADO DI ATTENUARE LE SOLLECITAZIONI TRASMESSE DAL TERRENO AGLI EDIFICI DURANTE UN EVENTO SISMICO, FILTRANDO LE FREQUENZE MAGGIORMENTE DANNOSE. GENERALMENTE, TRA LE DIVERSE ATTIVITA' SISMICHE, LE STRONG MOTION RISULTANO ESSERE LE PIU' DANNOSE SUI FABBRICATI IN QUANTO CARATTERIZZATE DA VIBRAZIONI CON AMPIEZZA E PERIODO TALI DA PRODURRE DANNI SU AMBIENTE E INFRASTRUTTURE: AMPIEZZA: 0.001 G ? 1 G; FREQUENZA: 0.06 HZ ? 25 HZ. VERRA' DUNQUE STUDIATA LA CONFIGURAZIONE DEL DISPOSITIVO CONDUCENDO, SUCCESSIVAMENTE, ANALISI STATICHE E DINAMICHE SUL PEZZO, PER ANALIZZARNE E VERIFICARNE IL COMPORTAMENTO. NELLA FATTISPECIE, DOPO AVER IPOTIZZATO UNA CONFIGURAZIONE PRELIMINARE DEL DISPOSITIVO, SI VERIFICHERA' LA RISPOSTA DELLO STESSO SOTTOPOSTO A SOLLECITAZIONI DI TIPO STATICHE INCREMENTATE GRADUALMENTE FINO AL RAGGIUNGIMENTO DELLE CONDIZIONI DI SNERVAMENTO DEL CAVO D'ACCIAIO. INOLTRE, VERRANNO ANALIZZATE LE DEFORMAZIONI INDOTTE SULL'ELASTOMERO, FUNZIONE DEL TIPO DI POLIMERO DA IMPIEGARE DURANTE LE ANALISI STATICHE E DINAMICHE. LE DEFORMAZIONI INDOTTE SULL'ELASTOMERO DIPENDERANNO DAL TIPO DI POLIMERO UTILIZZATO, CHE SARA' PERTANTO OGGETTO DI STUDIO UNO STUDIO SIMULATO, I CUI RISULTATI ATTESI DOVRANNO POI ESSERE CONFERMATI DALLE PROVE SPERIMENTALI CONDOTTE DAI LABORATORI DI PROVE SUI MATERIALI DELL'UNIVERSITA' DELLA BASILICATA. IN ULTIMO SARA' CONDOTTO UNO STUDIO DEGLI EFFETTI DISSIPATIVI LEGATI ALLA TIPOLOGIA DI SISTEMA DI SMORZAMENTO/ASSORBIMENTO DELLE SOLLECITAZIONI PREVISTE. ULTIMATA LA FASE DI INGEGNERIZZAZIONE DEL PROTOTIPO SARA' POSSIBILE LA REALIZZAZIONE DEL DISPOSITIVO PROTOTIPALE, AD OPERA DELLA DITTA CNC FACTORY. UNA VOLTA COSTRUITO, IL PROTOTIPO VERRA' MONTATO SU UN PROVINO PER LA PROVA DI CARATTERIZZAZIONE DEL PEZZO E PER LE PROVE SU TAVOLA VIBRANTE, CHE VERRANNO ESEGUITI DAI SUCCITATI LABORATORI UNIVERSITARI. LA TAVOLA SOTTOPORRA' IL PROVINO A MOVIMENTI OSCILLATORI, RENDENDO POSSIBILE L'OSSERVAZIONE DEL COMPORTAMENTO DINAMICO DELLE DEFORMAZIONI DELLA STRUTTURA. SARANNO, QUINDI, OSSERVABILI I FENOMENI LEGATI AL FILTRAGGIO DELLE FREQUENZE AL CONTROLLO DEI PERIODI DI OSCILLAZIONE DELLE STRUTTURE ALLE CURVE DI ISTERESI DI DISSIPAZIONE ENERGETICA DEL DISPOSITIVO, DI EFFETTI DEL SECONDO ORDINE E DI FENOMENI DI FATICA DEI MATERIALI. SARANNO, INOLTRE, REGISTRATI I DATI SPERIMENTALI CHE CONSENTIRANNO LA MODELLIZZAZIONE, LA CARATTERIZZAZIONE, LA CATALOGAZIONE E L'IMPLEMENTAZIONE SERIALE DEL DISPOSITIVO SU SCALA INDUSTRIALE. ALLA FASE SPERIMENTALE SEGUIRA' LA FASE DI CALCOLO IN CUI, IL DISPOSITIVO INSERITO OPPORTUNAMENTE IN STRUTTURE REALI, CON LE CARATTERISTICHE PROPRIE, GIA' TESTATE NELLA FASE SPERIMENTALE, POTRA' ESPRIMERE PIENAMENTE, TUTTE LE POTENZIALITA' DEL SISTEMA, IL SOFTWARE DI RIFERIMENTO A LIVELLO DI ECCELLENZA MONDIALE CHE SARA' UTILIZZATO PER VERIFICARE SU MODELLI STRUTTURALI DI EDIFICI REALI L'EFFICACIA DEL SISTEMA SARA' L'ASI CON ANALISI DINAMICHE NON LINEARI UTILIZZANDO IL CODICE DI CALCOLO AEM (APPLIED ELEMENT METHOD). INFINE, TERMINATA LA FASE DI IMPLEMENTAZIONE SARA' POSSIBILE PROCEDERE CON LA PROGETTAZIONE PRODUTTIVA. DETERMINATO L'OGGETTO FINALE SARA' IMPORTANTE STUDIARE I PROGETTI DI ASSEMBLAGGIO, DALL'ORIGINE FINO ALL'INIZIO DELLA PRODUZIONE. LA CAPACITA' DI SFRUTTARE I DATI 3D DEI PRODOTTI E DELLE RISORSE AGEVOLERA' LA VALIDAZIONE, L'OTTIMIZZAZIONE E L'ALLESTIMENTO VIRTUALE DEL PROCESSO PRODUTTIVO, RIDUCENDO I TEMPI DI AVVIO E AUMENTANDO LA QUALITA' DELLA PRODUZIONE, LO STUDIO SARA' CONDOTTO DALLA DITTA MOSAIC. IL PROCESS SIMULATE PERMETTERA' DI VERIFICARE LA FATTIBILITA' DEL PROCESSO DI ASSEMBLAGGIO, CONVALIDANDO LE CARATTERISTICHE DI RAGGIUNGIBILITA', PROSSIMITA' E COLLISIONI, GRAZIE ALLA SIMULAZIONE GLOBALE DELL'INTERO PROCESSO DI ASSEMBLAGGIO DEL PRODOTTO E DEGLI STRUMENTI NECESSARI.</t>
         </is>
       </c>
       <c r="CR2" t="inlineStr">
         <is>
-          <t>DIRITTI DI PRIVATIVA NON DICHIARATI COME REQUISITO DELLA STARTUP</t>
+          <t>LA SOCIETA' E' LICENZIATARIA DEL BREVETTO INDUSTRIALE N. 102017000099508 SISTEMA ANTISISMICO STRUTTURALE A DISSIPAZIONE DI ENERGIA CON CONTROVENTI PRETENSIONATI IN ACCIAIO OTTENUTO CON ADOZIONE DI GIUNTO ANTISISMICO CON ELASTOMERO</t>
         </is>
       </c>
       <c r="CS2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;?xml version="1.0"?&gt;
-&lt;dichiarazione xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance"&gt;&lt;info-dichiarazione&gt;&lt;codice&gt;01038800148-20251014171044&lt;/codice&gt;&lt;/info-dichiarazione&gt;&lt;info-schema&gt;&lt;tipo&gt;startup&lt;/tipo&gt;&lt;versione&gt;2&lt;/versione&gt;&lt;data-compilazione&gt;2025-10-14T17:06:22&lt;/data-compilazione&gt;&lt;/info-schema&gt;&lt;impresa&gt;&lt;codice-fiscale&gt;01038800148&lt;/codice-fiscale&gt;&lt;denominazione&gt;WIDE VR S.R.L.&lt;/denominazione&gt;&lt;/impresa&gt;&lt;informazioni&gt;&lt;logo&gt;&lt;extension&gt;&lt;/extension&gt;&lt;b64&gt;[ARCHIVED_IN_IMG_BB]&lt;/b64&gt;&lt;/logo&gt;&lt;stadio&gt;&lt;cod&gt;S3&lt;/cod&gt;&lt;decod&gt;&lt;en&gt;Launch&lt;/en&gt;&lt;it&gt;Sul mercato&lt;/it&gt;&lt;/decod&gt;&lt;/stadio&gt;&lt;presentazione&gt;&lt;descrizione&gt;&lt;en&gt;Wide VR is specialized in cutting-edge 3D solutions. We have developed several projects for international clients including Nike, Mapei and Italtherm. Wide VR presents Vshop, the first subscription-based platform for the automated creation of photorealistic quality virtual shops compatible with any e-commerce platform. Vshop solves the problem of low conversions in e-commerce due to a product experience limited by the use of photography. Virtual shops can be created from templates designed for different market niches including fashion, accessories and design. Spaces are navigated via the web with a quality close to realism, thanks to proprietary software based on an innovative pipeline, which combines new technologies including high poly 3D conversion and AI. The subscription-based business model provides economic plans that make the solution scalable.&lt;/en&gt;&lt;it&gt;Wide VR è una startup specializzata in soluzioni 3D cutting-edge. Abbiamo realizzato diversi progetti per clienti internazionali tra cui Nike, Mapei e Italtherm. Wide VR presenta Vshop, la prima piattaforma ad abbonamento per la creazione automatizzata di shop virtuali in qualità fotorealistica compatibili con qualunque piattaforma e-commerce. Vshop risolve il problema delle scarse conversioni in ambito e-commerce dovute ad un'esperienza del prodotto limitata dall'uso della fotografia. È possibile creare shop virtuali a partire da template pensati per diverse nicchie di mercato tra cui moda, accessori e design. La navigazione degli spazi avviene via web con una qualità vicina al realismo, grazie ad un software proprietario basato su una pipeline innovativa, che combina nuove tecnologie tra cui la conversione 3D high poly e L'AI. Il modello di business ad abbonamento prevede piani economici che rendono la soluzione scalabile.&lt;/it&gt;&lt;/descrizione&gt;&lt;/presentazione&gt;&lt;contatti&gt;&lt;email&gt;edoardo@widevr.eu&lt;/email&gt;&lt;facebook&gt;Facebook.com/widemilan&lt;/facebook&gt;&lt;linkedin&gt;https://www.linkedin.com/company/wide-vr/&lt;/linkedin&gt;&lt;youtube&gt;https://youtube.com/@widevr5265&lt;/youtube&gt;&lt;/contatti&gt;&lt;settore&gt;&lt;tag&gt;RealtaVirtuale&lt;/tag&gt;&lt;macro-settore&gt;&lt;cod&gt;MS9&lt;/cod&gt;&lt;decod&gt;&lt;en&gt;E-commerce&lt;/en&gt;&lt;it&gt;E-commerce&lt;/it&gt;&lt;/decod&gt;&lt;/macro-settore&gt;&lt;/settore&gt;&lt;prodotto&gt;&lt;stato-prodotto&gt;&lt;cod&gt;P3&lt;/cod&gt;&lt;decod&gt;&lt;en&gt;Ready&lt;/en&gt;&lt;it&gt;Pronto&lt;/it&gt;&lt;/decod&gt;&lt;/stato-prodotto&gt;&lt;descrizione-prodotto&gt;&lt;en&gt;Vshop is the first subscription-based platform for the automated creation of photorealistic quality virtual shops compatible with any e-commerce platform. Vshop solves the problem of low conversions in e-commerce due to a product experience limited by the use of photography. Virtual shops can be created from templates designed for different market niches including fashion, accessories and design. Spaces are navigated via the web with a quality close to realism, thanks to proprietary software based on an innovative pipeline, which combines new technologies including high poly 3D conversion and AI. The subscription-based business model provides economic plans that make the solution scalable.&lt;/en&gt;&lt;it&gt;Vshop è la prima piattaforma ad abbonamento per la creazione automatizzata di shop virtuali in qualità fotorealistica compatibili con qualunque piattaforma e-commerce. Vshop risolve il problema delle scarse conversioni in ambito e-commerce dovute ad un'esperienza del prodotto limitata dall'uso della fotografia. È possibile creare shop virtuali a partire da template pensati per diverse nicchie di mercato tra cui moda, accessori e design. La navigazione degli spazi avviene via web con una qualità vicina al realismo, grazie ad un software proprietario basato su una pipeline innovativa, che combina nuove tecnologie tra cui la conversione 3D high poly e L'AI. Il modello di business ad abbonamento prevede piani economici che rendono la soluzione scalabile.&lt;/it&gt;&lt;/descrizione-prodotto&gt;&lt;/prodotto&gt;&lt;team&gt;&lt;stato-team&gt;&lt;cod&gt;T4&lt;/cod&gt;&lt;decod&gt;&lt;en&gt;Defined&lt;/en&gt;&lt;it&gt;Completo&lt;/it&gt;&lt;/decod&gt;&lt;/stato-team&gt;&lt;soggetto&gt;&lt;occupazione-startup-team&gt;&lt;en&gt;Edoardo Graziadei, CEO&lt;/en&gt;&lt;it&gt;Edoardo Graziadei, CEO&lt;/it&gt;&lt;/occupazione-startup-team&gt;&lt;livello-titolo-studio&gt;&lt;cod&gt;LTS3&lt;/cod&gt;&lt;decod&gt;&lt;en&gt;Bachelor's degree&lt;/en&gt;&lt;it&gt;Laurea triennale&lt;/it&gt;&lt;/decod&gt;&lt;/livello-titolo-studio&gt;&lt;fascia-eta&gt;&lt;cod&gt;FE4&lt;/cod&gt;&lt;decod&gt;&lt;en&gt;30-34&lt;/en&gt;&lt;it&gt;30-34&lt;/it&gt;&lt;/decod&gt;&lt;/fascia-eta&gt;&lt;descrizione-ruolo-team&gt;&lt;en&gt;CEO and co-founder&lt;/en&gt;&lt;it&gt;CEO e co-founder&lt;/it&gt;&lt;/descrizione-ruolo-team&gt;&lt;/soggetto&gt;&lt;soggetto&gt;&lt;occupazione-startup-team&gt;&lt;en&gt;Andrea Zardin, COO&lt;/en&gt;&lt;it&gt;Andrea Zardin, COO&lt;/it&gt;&lt;/occupazione-startup-team&gt;&lt;livello-titolo-studio&gt;&lt;cod&gt;LTS1&lt;/cod&gt;&lt;decod&gt;&lt;en&gt;Secondary education (lower or upper)&lt;/en&gt;&lt;it&gt;Scuola media o superiore&lt;/it&gt;&lt;/decod&gt;&lt;/livello-titolo-studio&gt;&lt;fascia-eta&gt;&lt;cod&gt;FE5&lt;/cod&gt;&lt;decod&gt;&lt;en&gt;35-39&lt;/en&gt;&lt;it&gt;35-39&lt;/it&gt;&lt;/decod&gt;&lt;/fascia-eta&gt;&lt;descrizione-ruolo-team&gt;&lt;en&gt;COO and co-founder&lt;/en&gt;&lt;it&gt;COO e co-founder&lt;/it&gt;&lt;/descrizione-ruolo-team&gt;&lt;/soggetto&gt;&lt;/team&gt;&lt;mercato&gt;&lt;area-geografica&gt;&lt;cod&gt;A4&lt;/cod&gt;&lt;decod&gt;&lt;en&gt;Italy&lt;/en&gt;&lt;it&gt;Italia&lt;/it&gt;&lt;/decod&gt;&lt;/area-geografica&gt;&lt;area-geografica-italia&gt;&lt;cod&gt;08&lt;/cod&gt;&lt;decod&gt;&lt;en&gt;EMILIA-ROMAGNA&lt;/en&gt;&lt;it&gt;EMILIA-ROMAGNA&lt;/it&gt;&lt;/decod&gt;&lt;/area-geografica-italia&gt;&lt;area-geografica-italia&gt;&lt;cod&gt;03&lt;/cod&gt;&lt;decod&gt;&lt;en&gt;LOMBARDIA&lt;/en&gt;&lt;it&gt;LOMBARDIA&lt;/it&gt;&lt;/decod&gt;&lt;/area-geografica-italia&gt;&lt;area-geografica-italia&gt;&lt;cod&gt;09&lt;/cod&gt;&lt;decod&gt;&lt;en&gt;TOSCANA&lt;/en&gt;&lt;it&gt;TOSCANA&lt;/it&gt;&lt;/decod&gt;&lt;/area-geografica-italia&gt;&lt;area-geografica-estero&gt;&lt;cod&gt;11&lt;/cod&gt;&lt;decod&gt;&lt;en&gt;European Union&lt;/en&gt;&lt;it&gt;Unione europea&lt;/it&gt;&lt;/decod&gt;&lt;/area-geografica-estero&gt;&lt;area-geografica-estero&gt;&lt;cod&gt;41&lt;/cod&gt;&lt;decod&gt;&lt;en&gt;Northern America&lt;/en&gt;&lt;it&gt;America settentrionale&lt;/it&gt;&lt;/decod&gt;&lt;/area-geografica-estero&gt;&lt;canale-di-vendita&gt;&lt;cod&gt;C1&lt;/cod&gt;&lt;decod&gt;&lt;en&gt;Directly&lt;/en&gt;&lt;it&gt;Direttamente&lt;/it&gt;&lt;/decod&gt;&lt;/canale-di-vendita&gt;&lt;/mercato&gt;&lt;business-model&gt;&lt;descrizione-business-model&gt;&lt;en&gt;Saas with monthly subscrption&lt;/en&gt;&lt;it&gt;Saas con abbonamento mensile&lt;/it&gt;&lt;/descrizione-business-model&gt;&lt;/business-model&gt;&lt;concorrenza&gt;&lt;descrizione-concorrenza&gt;&lt;en&gt;In Italy, competitors use low-end technologies such as 360° videos, while we work across multiple verticals in real-time 3D with dedicated pipelines.&lt;/en&gt;&lt;it&gt;In Italia i competitor usano tecnologie poco avanzate come i video 360, noi lavoriamo sui vari verticali in real-time 3D con pipeline specifiche.&lt;/it&gt;&lt;/descrizione-concorrenza&gt;&lt;/concorrenza&gt;&lt;innovazione&gt;&lt;proprieta-intellettuale&gt;false&lt;/proprieta-intellettuale&gt;&lt;descrizione-proprieta-intellettuale&gt;&lt;en&gt;Real-time 3D con output fotorealistico integrato con AI.&lt;/en&gt;&lt;it&gt;Real-time 3D with photorealistic output, fully integrated with AI.&lt;/it&gt;&lt;/descrizione-proprieta-intellettuale&gt;&lt;/innovazione&gt;&lt;finanze&gt;&lt;non-disponibile&gt;true&lt;/non-disponibile&gt;&lt;/finanze&gt;&lt;associazione&gt;&lt;iscrizione&gt;false&lt;/iscrizione&gt;&lt;/associazione&gt;&lt;incubatori&gt;&lt;incubatore-accelerato&gt;false&lt;/incubatore-accelerato&gt;&lt;/incubatori&gt;&lt;/informazioni&gt;&lt;/dichiarazione&gt;
-</t>
+          <t>&lt;?xml version="1.0"?&gt;
+&lt;dichiarazione xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance"&gt;&lt;info-dichiarazione&gt;&lt;codice&gt;00977110949-20240618173252&lt;/codice&gt;&lt;/info-dichiarazione&gt;&lt;info-schema&gt;&lt;tipo&gt;startup&lt;/tipo&gt;&lt;versione&gt;2&lt;/versione&gt;&lt;data-compilazione&gt;2024-06-18T17:31:31&lt;/data-compilazione&gt;&lt;/info-schema&gt;&lt;impresa&gt;&lt;codice-fiscale&gt;00977110949&lt;/codice-fiscale&gt;&lt;denominazione&gt;MEDITERRANEA SOCIETA' A RESPONSABILITA' LIMITATA SEMPLIFICATA&lt;/denominazione&gt;&lt;/impresa&gt;&lt;informazioni&gt;&lt;logo&gt;&lt;extension&gt;&lt;/extension&gt;&lt;b64&gt;[ARCHIVED_IN_IMG_BB]&lt;/b64&gt;&lt;/logo&gt;&lt;stadio&gt;&lt;cod&gt;S2&lt;/cod&gt;&lt;decod&gt;&lt;en&gt;Development&lt;/en&gt;&lt;it&gt;Sviluppo&lt;/it&gt;&lt;/decod&gt;&lt;/stadio&gt;&lt;presentazione&gt;&lt;descrizione&gt;&lt;en&gt;Presentation of the company and related activities&amp;#x0D;
+&amp;#x0D;
+The company Mediterranea s.r.l.s., innovative startup, patent licensee for industrial invention G.A.E (Elastomeric Seismic Joint), fundamental component of the LE.A.D. (Dissipative Seismic Bindings), started the activity on 16/01/2020.&amp;#x0D;
+The corporate purpose consists of specialized work on buildings in steel, reinforced concrete and masonry.&amp;#x0D;
+Specifically, the processes consist of a structural system of ligation of civil structures framed in steel, reinforced concrete and masonry (LE.A.D.), which allows to modify and improve or adapt the response of the structural organism in the event of an earthquake.&amp;#x0D;
+The whole system is based on the creation of "dissipative" bracing consisting of tie rods connected through G.A.E. to the supporting structure, these joints have the ability to dissipate energy.&amp;#x0D;
+The particularity of the invention consists in the adoption of the aforementioned joints, defined as "Elastomeric Anti-Seismic Joints" (GAE), with high standardization to allow their assembly, in extremely short times, in a great variety of geometric configurations on the load-bearing structures of a building, in in order to adapt the structures to the dictates of the current national seismic legislation.&amp;#x0D;
+Mediterranea s.r.l.s will have as its purpose the development, production and marketing and installation of the LE.A.D. of which the elastomeric joint G.A.E. the subject of the patent is an essential part.&amp;#x0D;
+The Mediterranea company is composed of: Arch. Pier Luigi Pacitti, Ing. Antonio Libero Bucci.&amp;#x0D;
+Arch. Pier Luigi Pacitti and Eng. Antonio Libero Bucci have gained a deep experience in the technical field, with particular regard in the field of architectural design and anti-seismic renovation of buildings, for the methods of cataloging and survey of environmental detractors and of verification of urban planning tools.&amp;#x0D;
+Specifically, the over twenty years of experience acquired in the procedural field is highlighted with particular regard to the bureaucratic / administrative process of design practices, from authorizations, to environmental, urban planning, energy saving, anti-seismic, technological and electrical laws.&amp;#x0D;
+Eng. Antonio Libero Bucci, co-owner of the patent and co-inventor of the anti-seismic system, graduated in Civil Engineering from the University of Rome La Sapienza in July 1987, with thirty years of experience in the field of building renovation, with particular activity in the field of adaptation and&amp;#x0D;
+seismic improvement of buildings The system of anti-seismic dissipative ties is based on the realization of a&amp;#x0D;
+"dissipative" bracing consisting of tie rods connected to the structure through special joints that have the ability to dissipate energy thanks to elements in&amp;#x0D;
+elastomer.&amp;#x0D;
+&amp;#x0D;
+&amp;#x0D;
+Mediterrranea S.r.L.s. Viale dei Pentri 117 / a 86170 Isernia (IS)&amp;#x0D;
+Viale dei Pentri 117 / a 86170 Isernia tel / fax 0865 299759 - VAT number 00977110949&amp;#x0D;
+studio.mediterrranea@gmail.com www.mediterrenea-lide.com&amp;#x0D;
+&amp;#x0D;
+V / 2-2022&lt;/en&gt;&lt;it&gt;Presentazione aziendale e delle attività correlate&amp;#x0D;
+&amp;#x0D;
+La società Mediterranea s.r.l.s., startup innovativa, licenziataria di brevetto per invenzione industriale G.A.E (Giunto Antisismico Elastomerico) componente fondamentale del sistema LE.A.D. (LEgature Antisismiche Dissipative), ha iniziato l’attività in data 16/01/2020.&amp;#x0D;
+L’oggetto sociale consiste in lavorazioni specializzate su edifici in acciaio, cemento armato e muratura.&amp;#x0D;
+Nello specifico, le lavorazioni consistono in un sistema strutturale di legatura di strutture civile intelaiate in acciaio, c.l.s armato e muratura (LE.A.D.), che permette di modificare e migliorare o adeguare la risposta dell'organismo strutturale in caso di sisma.&amp;#x0D;
+Tutto il sistema è imperniato sulla realizzazione di controventi "dissipativi" costituiti da tiranti collegati attraverso Giunti Antisismici Elastomerici G.A.E. alla struttura portante, tali giunti hanno capacità di dissipare energia.&amp;#x0D;
+La particolarità dell'invenzione consiste nella adozione dei predetti giunti, definiti "Giunti Antisismici Elastomerici" (GAE), ad elevata standardizzazione per consentirne il montaggio, in tempi estremamente rapidi, in una grande varietà di configurazioni geometriche sulle strutture portanti di un edificio, in modo da adeguare le strutture ai dettami della vigente normativa sismica nazionale.&amp;#x0D;
+La Mediterranea s.r.l.s avrà come scopo lo sviluppo, la produzione e la commercializzazione e l’installazione del sistema LE.A.D. di cui il giunto elastomerico G.A.E. oggetto del brevetto è parte essenziale.&amp;#x0D;
+La società Mediterranea, è composta da: Arch. Pier Luigi Pacitti,  Ing. Antonio Libero Bucci.&amp;#x0D;
+L’Arch. Pier Luigi Pacitti e l’Ing. Antonio Libero Bucci hanno maturato una profonda esperienza nel campo tecnico, con particolare riguardo nel campo della progettazione architettonica e della ristrutturazione antisismica degli edifici, per i metodi di catalogazione e rilievo di detrattori ambientali e di verifica di strumenti urbanistici.&amp;#x0D;
+Si evidenzia, nello specifico, l’ultraventennale esperienza acquisita nel campo procedurale con particolare riguardo per quel che riguarda l'iter burocratico/amministrativo delle pratiche progettuali, dalle autorizzazioni, alle leggi ambientali, urbanistiche, sul risparmio energetico, antisismiche, tecnologiche ed elettriche.&amp;#x0D;
+L’Ing. Antonio Libero Bucci contitolare del brevetto e coinventore del sistema antisismico, laureatosi in Ingegneria Civile Edile presso l’Università degli Studi di Roma La Sapienza nel Luglio 1987, con esperienza trentennale nel campo della ristrutturazione edilizia , con particolare attività nel campo dell’adeguamento e&amp;#x0D;
+miglioramento sismico degli edifici Il sistema di legature antisismiche dissipative si basa sulla realizzazione di legature a&amp;#x0D;
+controventi "dissipativi" costituiti da tiranti collegati alla struttura attraverso particolari giunti che hanno la capacità di dissipare energia grazie ad elementi in&amp;#x0D;
+elastomero.&amp;#x0D;
+&amp;#x0D;
+&amp;#x0D;
+Mediterrranea S.r.L.s. Viale dei Pentri 117/a 86170 Isernia (IS)&amp;#x0D;
+Viale dei Pentri 117/a 86170 Isernia tel/fax 0865 299759 – p.iva 00977110949&amp;#x0D;
+studio.mediterrranea@gmail.com www.mediterrenea-lide.com&amp;#x0D;
+&amp;#x0D;
+V/2-2022&lt;/it&gt;&lt;/descrizione&gt;&lt;/presentazione&gt;&lt;contatti&gt;&lt;email&gt;studio.mediterrranea@gmail.com&lt;/email&gt;&lt;/contatti&gt;&lt;settore&gt;&lt;tag&gt;architettura&lt;/tag&gt;&lt;tag&gt;Antisismico&lt;/tag&gt;&lt;tag&gt;Ingegneria&lt;/tag&gt;&lt;macro-settore&gt;&lt;cod&gt;MS10&lt;/cod&gt;&lt;decod&gt;&lt;en&gt;Services&lt;/en&gt;&lt;it&gt;Servizi&lt;/it&gt;&lt;/decod&gt;&lt;/macro-settore&gt;&lt;/settore&gt;&lt;prodotto&gt;&lt;stato-prodotto&gt;&lt;cod&gt;P2&lt;/cod&gt;&lt;decod&gt;&lt;en&gt;Prototype/beta version&lt;/en&gt;&lt;it&gt;Prototipo/versione beta&lt;/it&gt;&lt;/decod&gt;&lt;/stato-prodotto&gt;&lt;descrizione-prodotto&gt;&lt;en&gt;The particularity of the invention consists precisely in the adoption of the aforementioned joints, called anti-seismic joints with elastomers (indicated by the acronym "GAE").&amp;#x0D;
+This joint is highly standardized to allow its assembly in extremely short times, in a great variety of geometric configurations of the load bearing structures of a building.&amp;#x0D;
+The GAE is made up of a specially designed cylindrical joint which houses the stringing head of a threaded rod tie rod. The adoption of threaded rods allows to minimize the overall dimensions of the clamping system and allows, by simply screwing a nut, to give a pretensioning of the tie rod, which will be calibrated using torque wrenches. The tie head housing system provides for the interposition of a Newton-type elastomeric element with an elasto-plastic characterization, which gives it the ability to dissipate energy.&amp;#x0D;
+By dosing the pre-tensioning of the tie rod and the elastic response of the elastomer cartridge housed in the joint, it is possible to "modulate" the reaction of the tie rod and "pilot" the response in seismic conditions of the entire load-bearing structure of the building.&amp;#x0D;
+In summary, the characteristics of the GAE are:&amp;#x0D;
+1. Dissipative capacity modifiable according to needs;&amp;#x0D;
+2. Ease of assembly&amp;#x0D;
+3. Easy and inexpensive restoration following an earthquake and periodic maintenance, thanks to the replacement of the elastomeric element only housed in the joint (cartridge);&amp;#x0D;
+4. Limited dimensions and weight for easy transport and assembly;&amp;#x0D;
+5. Reduced assembly times.&amp;#x0D;
+For the exploitation of patent technology, analytical studies must be undertaken in order to validate and pursue system improvements; the compulsory stages of the prototype development necessary for the validation of the system by the Superior Council of Public Works have been identified.&amp;#x0D;
+The company is the beneficiary of the loan of Euro 131,742.88 obtained through the European PATENT + loan granted by INVITALIA, a national company for the attraction of investments and the development of a SPA company.&amp;#x0D;
+The key step of the procedural process will be the creation of an experimental prototype, tested on a vibrating table and analyzed in order to proceed with modeling.&amp;#x0D;
+Therefore, the services necessary for the development and subsequent validation of the system are:&amp;#x0D;
+1) Analysis and industrialization of the device, which includes:&amp;#x0D;
+a) Study, design and engineering of the prototype:&amp;#x0D;
+i) Modeling and engineering;&amp;#x0D;
+ii) Static and dynamic modeling analysis on the device;&amp;#x0D;
+iii) Dissipative effects analysis;&amp;#x0D;
+iv) Frequency filtering analysis&amp;#x0D;
+v) Analysis of the hysteresis curves and the dissipative capacity of the device&amp;#x0D;
+vi) Analysis of the resonance factors and development of configurations that can avoid situations that cannot be controlled&amp;#x0D;
+vii) Study of the fatigue of the elements involved&amp;#x0D;
+viii) Design of the production process&amp;#x0D;
+This study will be conducted by a company specializing in the study of mechanical cushioning devices.&amp;#x0D;
+2) Realization of the prototype, will be carried out by the CNC Factory company specialized in the realization and production of mechanical parts.&amp;#x0D;
+3) Experimental verification of both the qualification of the piece and its application to a structure specially made on a vibrating table.&amp;#x0D;
+The study will be conducted by the materials testing laboratory of the University of Basilicata.&amp;#x0D;
+4) Modeling and structural calculation on models of real buildings in different structural configurations, stressed with different accelerograms representative of real earthquakes, with non-linear dynamic analysis, as required for such devices in the legislation.&amp;#x0D;
+This study will be conducted by ASI Europa, a leading company specializing in AEM structural calculation.&amp;#x0D;
+5) Production, standardization of the process (including the structural calculation procedure and application studies on real buildings), and marketing of the device.&amp;#x0D;
+6) Implementation&amp;#x0D;
+7) Periodic maintenance of the devices&amp;#x0D;
+Specifically, the purpose of the study will be to prove that the system is able to attenuate the stresses transmitted from the ground to buildings during a seismic event, filtering the most damaging frequencies.&amp;#x0D;
+Generally, among the various seismic activities, strong motion are the most harmful on buildings as they are characterized by vibrations with amplitude and period such as to produce damage to the environment and infrastructure:&amp;#x0D;
+• Amplitude: 0.001 g ÷ 1 g;&amp;#x0D;
+• Frequency: 0.06 Hz ÷ 25 Hz.&amp;#x0D;
+The configuration of the device will therefore be studied, subsequently carrying out static and dynamic analyzes on the piece, to analyze and verify its behavior.&amp;#x0D;
+In this case, after having assumed a preliminary configuration of the device, the response of the device will be verified subjected to static stresses gradually increased until the yield conditions of the steel cable are reached. Furthermore, the deformations induced on the elastomer will be analyzed, depending on the type of polymer to be used during the static and dynamic analyzes. The deformations induced on the elastomer will depend on the type of polymer used, which will therefore be the subject of a simulated study, the expected results of which must then be confirmed by experimental tests.&amp;#x0D;
+Finally, a study of the dissipative effects related to the type of damping / absorption system of the foreseen stresses will be carried out.&amp;#x0D;
+Once the prototype engineering phase has been completed, it will be possible to create the prototype device.&amp;#x0D;
+Once built, the prototype and cataloged in different configurations and types, will be mounted on a model for the characterization test of the piece and for the vibrating table tests, which will be performed by accredited specialized laboratories and / or research institutes, specifically University of Basilicata, materials testing laboratory.&amp;#x0D;
+The table will subject the specimen to oscillatory movements, making it possible to observe the dynamic behavior of the deformations of the structure.&amp;#x0D;
+Therefore, the phenomena related to the filtering of frequencies to the control of the periods of oscillation of the structures to the hysteresis curves of energy dissipation of the device, of second order effects and of material fatigue phenomena, will be observable. The experimental data will also be recorded that will allow the modeling, characterization, cataloging and serial implementation of the device on an industrial scale.&amp;#x0D;
+The experimental phase will be followed by the calculation phase in which the device properly inserted in real structures, with its own characteristics, already tested in the experimental phase, will be able to fully express all the potential of the system.&amp;#x0D;
+Finally, once the implementation phase is complete, it will be possible to proceed with the production design.&amp;#x0D;
+Once the final object has been determined, it will be important to study the assembly projects, from the origin to the start of production.&amp;#x0D;
+The ability to leverage 3D product and asset data will facilitate the validation, optimization and virtual setup of the production process, reducing start-up times and increasing production quality.&amp;#x0D;
+The Process Simulate will allow to verify the feasibility of the assembly process, validating the characteristics of reachability, proximity and collisions, thanks to the global simulation of the entire assembly process of the product and the necessary tools.&amp;#x0D;
+Automatic creation of assembly sequences will improve the productivity of the planning process. Tools such as sections, measurements and collision detection will allow you to check and optimize assembly situations in detail.&amp;#x0D;
+Finally, in order to proceed with the start of production and marketing, the technical-administrative endorsement of the LE.A.D. system will be required. by the Higher Council of Public Works.&amp;#x0D;
+The Mediterranea company considers it essential to find financing partners or leading companies in the sector of seismic adaptation and improvement of buildings, to complement its corporate action, in order to make the most of the strong opportunities offered by the sector.&amp;#x0D;
+A study was conducted on the state of the art of the seismic dissipator market.&amp;#x0D;
+The main competitors were identified, the size of the seismic vulnerability of the Italian built heritage was quantified.&amp;#x0D;
+These cognitive actions made it possible to estimate the potential market and to identify the main critical issues for the time to market.&amp;#x0D;
+In particular, the barriers to market entry were analyzed and the necessary actions were developed to overcome them.&amp;#x0D;
+Furthermore, given the nature of a market strongly oriented towards the research and development of innovative solutions, it is believed that the time factor plays a decisive role in the success of the product on the market.&amp;#x0D;
+&amp;#x0D;
+&amp;#x0D;
+Mediterrranea S.r.L.s. Viale dei Pentri 117 / a 86170 Isernia (IS)&amp;#x0D;
+Viale dei Pentri 117 / a 86170 Isernia tel / fax 0865 299759 - VAT number 00977110949&amp;#x0D;
+studio.mediterrranea@gmail.com www.mediterrenea-lide.com&amp;#x0D;
+&amp;#x0D;
+V / 1-2020&lt;/en&gt;&lt;it&gt;La particolarità dell'invenzione consiste proprio nell’adozione dei predetti giunti, denominati giunti antisismici con elastomeri (indicato dall'acronimo “GAE”).&amp;#x0D;
+Tale giunto presenta elevata standardizzazione per consentirne il montaggio in tempi estremamente rapidi, in una grande varietà di configurazioni geometriche delle strutture portanti di un edificio.&amp;#x0D;
+Il GAE è costituito da uno snodo cilindrico, appositamente concepito, che ospita la testa di tesatura di un tirante in barra filettata. L’adozione di barre filettate permette di contenere al minimo l’ingombro del sistema di serraggio e permette, tramite il semplice avvitamento di un dado, di conferire un pretensionamento del tirante, che verrà calibrato tramite chiavi dinamometriche. Il sistema di alloggiamento della testa tirante prevede l’interposizione di un elemento elastomerico di tipo Newton a caratterizzazione elasto-plastica, che conferisce la capacità di dissipare energia.&amp;#x0D;
+Andando a dosare il pretensionamento del tirante e la risposta elastica della cartuccia di elastomero alloggiata nel giunto si riesce a “modulare” la reazione del tirante ed a “pilotare” la risposta in condizioni sismiche dell’intera struttura portante dell’edificio.&amp;#x0D;
+In sintesi le caratteristiche del GAE sono:&amp;#x0D;
+1. Capacità dissipativa modificabile in funzione delle necessità;&amp;#x0D;
+2. Facilità di montaggio&amp;#x0D;
+3. Facilità ed economicità di ripristino a seguito di sisma e di manutenzione periodica, grazie alla sostituibilità del solo elemento elastomerico alloggiato nel giunto (cartuccia);&amp;#x0D;
+4. Dimensioni e peso contenuti per un agevole trasporto e montaggio;&amp;#x0D;
+5. Ridotti tempi di montaggio.&amp;#x0D;
+Per la valorizzazione della tecnologia brevettuale devono essere intrapresi studi analitici allo scopo di validare e perseguire miglioramenti del sistema; sono state individuate le tappe obbligatorie dello sviluppo prototipale necessarie alla vidimazione del sistema stesso da parte del Consiglio Superiore dei Lavori Pubblici.&amp;#x0D;
+La società è beneficiaria del finanziamento di Euro 131.742,88 ottenuto attraverso il bando europeo BREVETTI+ finanziamento concesso da INVITALIA azienda nazionale per l’attrazione degli investimenti e lo sviluppo d’impresa SPA.&amp;#x0D;
+Passaggio chiave dell’iter procedurale sarà, la realizzazione di un prototipo sperimentale, testato su tavola vibrante e analizzato in modo da procedere alla modellizzazione.&amp;#x0D;
+Quindi, i servizi necessari allo sviluppo e alla successiva validazione del sistema sono:&amp;#x0D;
+1) Analisi e industrializzazione dell’apparecchio, che include:&amp;#x0D;
+a) Studio, progettazione ed ingegnerizzazione del prototipo:&amp;#x0D;
+i) Modellazione e ingegnerizzazione;&amp;#x0D;
+ii) Analisi statiche e dinamiche modellistiche sul dispositivo;&amp;#x0D;
+iii) Analisi effetti dissipativi;&amp;#x0D;
+iv) Analisi del filtraggio delle frequenze&amp;#x0D;
+v) Analisi delle curve di isteresi e della capacità dissipativa dell’apparecchio&amp;#x0D;
+vi) Analisi dei fattori di risonanza e messa a punto di configurazioni che possano scongiurare situazioni non controllabili&amp;#x0D;
+vii) Studio della fatica degli elementi interessati&amp;#x0D;
+viii) Progettazione del processo produttivo&amp;#x0D;
+Tale studio verrà condotto da una società specializzata nello studio di dispositivi di ammortizzazione meccanica.&amp;#x0D;
+2) Realizzazione del prototipo, verrà eseguito dalla società CNC Factory specializzata nella realizzazione e produzione di pezzi meccanici.&amp;#x0D;
+3) Verifica sperimentale sia di qualificazione del pezzo che di applicazione dello stesso ad una struttura appositamente realizzata su tavola vibrante.&amp;#x0D;
+Lo studio verrà condotto dal laboratorio prove sui materiali dell’Università della Basilicata.&amp;#x0D;
+4) La modellizzazione ed il calcolo strutturale su modelli di edifici reali in diverse configurazioni strutturali, sollecitati con differenti accellerogrammi rappresentativi di terremoti reali, con analisi dinamica non lineare, come previsto per tali dispositivi in normativa.&amp;#x0D;
+Tale studio verrà condotto dalla società ASI Europa società leader specializzata nel calcolo strutturale AEM.&amp;#x0D;
+5) Messa in produzione, standardizzazione del processo (inclusa la procedura di calcolo strutturale e gli studi applicativi sugli edifici reali), e commercializzazione del dispositivo.&amp;#x0D;
+6) Messa in opera&amp;#x0D;
+7) Manutenzione periodica dei dispositivi&amp;#x0D;
+Nello specifico, scopo dello studio sarà provare che il sistema è in grado di attenuare le sollecitazioni trasmesse dal terreno agli edifici durante un evento sismico, filtrando le frequenze maggiormente dannose.&amp;#x0D;
+Generalmente, tra le diverse attività sismiche, le strong motion risultano essere le più dannose sui fabbricati in quanto caratterizzate da vibrazioni con ampiezza e periodo tali da produrre danni su ambiente e infrastrutture:&amp;#x0D;
+• Ampiezza: 0.001 g ÷ 1 g;&amp;#x0D;
+• Frequenza: 0.06 Hz ÷ 25 Hz.&amp;#x0D;
+Verrà dunque studiata la configurazione del dispositivo conducendo, successivamente, analisi statiche e dinamiche sul pezzo, per analizzarne e verificarne il comportamento.&amp;#x0D;
+Nella fattispecie, dopo aver ipotizzato una configurazione preliminare del dispositivo, si verificherà la risposta dello stesso sottoposto a sollecitazioni di tipo statiche incrementate gradualmente fino al raggiungimento delle condizioni di snervamento del cavo d’acciaio. Inoltre, verranno analizzate le deformazioni indotte sull’elastomero, funzione del tipo di polimero da impiegare durante le analisi statiche e dinamiche. Le deformazioni indotte sull’elastomero dipenderanno dal tipo di polimero utilizzato, che sarà pertanto oggetto di studio uno studio simulato, i cui risultati attesi dovranno poi essere confermati dalle prove sperimentali.&amp;#x0D;
+In ultimo sarà condotto uno studio degli effetti dissipativi legati alla tipologia di sistema di smorzamento/assorbimento delle sollecitazioni previste.&amp;#x0D;
+Ultimata la fase di ingegnerizzazione del prototipo sarà possibile la realizzazione del dispositivo prototipale.&amp;#x0D;
+Una volta costruito, il prototipo e catalogato in differenti configurazioni e tipologie, verrà montato su un modello per la prova di caratterizzazione del pezzo e per le prove su tavola vibrante, che verrà eseguita da laboratori specializzati accreditati e/o istituti di ricerca, nello specifico Università degli Studi della Basilicata, laboratorio di prove sui materiali.&amp;#x0D;
+La tavola sottoporrà il provino a movimenti oscillatori, rendendo possibile l'osservazione del comportamento dinamico delle deformazioni della struttura.&amp;#x0D;
+Saranno, quindi, osservabili i fenomeni legati al filtraggio delle frequenze al controllo dei periodi di oscillazione delle strutture alle curve di isteresi di dissipazione energetica del dispositivo, di effetti del secondo ordine e di fenomeni di fatica dei materiali. Saranno, inoltre, registrati i dati sperimentali che consentiranno la modellizzazione, la caratterizzazione, la catalogazione e l’implementazione seriale del dispositivo su scala industriale.&amp;#x0D;
+Alla fase sperimentale seguirà la fase di calcolo in cui, il dispositivo inserito opportunamente in strutture reali, con le caratteristiche proprie, già testate nella fase sperimentale, potrà esprimere pienamente, tutte le potenzialità del sistema.&amp;#x0D;
+Infine, terminata la fase di implementazione sarà possibile procedere con la progettazione produttiva.&amp;#x0D;
+Determinato l’oggetto finale sarà importante studiare i progetti di assemblaggio, dall'origine fino all'inizio della produzione.&amp;#x0D;
+La capacità di sfruttare i dati 3D dei prodotti e delle risorse agevolerà la validazione, l'ottimizzazione e l'allestimento virtuale del processo produttivo, riducendo i tempi di avvio e aumentando la qualità della produzione.&amp;#x0D;
+Il Process Simulate permetterà di verificare la fattibilità del processo di assemblaggio, convalidando le caratteristiche di raggiungibilità, prossimità e collisioni, grazie alla simulazione globale dell'intero processo di assemblaggio del prodotto e degli strumenti necessari.&amp;#x0D;
+La creazione automatica delle sequenze di assemblaggio consentirà di migliorare la produttività del processo di pianificazione. Strumenti quali sezioni, misurazioni e rilevazione delle collisioni permetteranno di verificare e ottimizzare in modo dettagliato le situazioni di assemblaggio.&amp;#x0D;
+Infine, per poter procedere con l’avvio della produzione e commercializzazione sarà necessaria la vidimazione tecnico-amministrativa del sistema LE.A.D. da parte del Consiglio Superiore dei Lavori Pubblici.&amp;#x0D;
+La società Mediterranea, ritiene indispensabile, la ricerca di soci finanziatori o società leader nel settore dell’adeguamento e miglioramento sismico dei fabbricati, da affiancare alla propria azione societaria, al fine di sfruttare al meglio le forti opportunità offerte dal settore.&amp;#x0D;
+E’ stato condotto uno studio, sullo stato dell’arte del mercato dei dissipatori sismici.&amp;#x0D;
+Sono stati individuati i principali competitor, è stata quantificata la dimensione della vulnerabilità sismica del patrimonio edificato italiano.&amp;#x0D;
+Tali azioni conoscitive hanno permesso di stimare il mercato potenziale e di individuare le principali criticità per il time to market.&amp;#x0D;
+In particolare, sono state analizzate le barriere all’ingresso del mercato e sono state elaborate le azioni necessarie per superarle.&amp;#x0D;
+Altresì, data la natura di un mercato fortemente orientato alla ricerca e sviluppo di soluzioni innovative, si ritiene che il fattore tempo giochi un ruolo determinante per il successo del prodotto sul mercato.&amp;#x0D;
+&amp;#x0D;
+&amp;#x0D;
+Mediterrranea S.r.L.s. Viale dei Pentri 117/a 86170 Isernia (IS)&amp;#x0D;
+Viale dei Pentri 117/a 86170 Isernia tel/fax 0865 299759 – p.iva 00977110949&amp;#x0D;
+studio.mediterrranea@gmail.com www.mediterrenea-lide.com&amp;#x0D;
+&amp;#x0D;
+V/1-2020&lt;/it&gt;&lt;/descrizione-prodotto&gt;&lt;/prodotto&gt;&lt;team&gt;&lt;stato-team&gt;&lt;cod&gt;T2&lt;/cod&gt;&lt;decod&gt;&lt;en&gt;Technical team complete&lt;/en&gt;&lt;it&gt;Completo solo lato tecnico&lt;/it&gt;&lt;/decod&gt;&lt;/stato-team&gt;&lt;soggetto&gt;&lt;occupazione-startup-team&gt;&lt;en&gt;engineer&lt;/en&gt;&lt;it&gt;Ingegnere&lt;/it&gt;&lt;/occupazione-startup-team&gt;&lt;livello-titolo-studio&gt;&lt;cod&gt;LTS4&lt;/cod&gt;&lt;decod&gt;&lt;en&gt;Master's degree or equivalent&lt;/en&gt;&lt;it&gt;Laurea magistrale/a ciclo unico/vecchio ordinamento&lt;/it&gt;&lt;/decod&gt;&lt;/livello-titolo-studio&gt;&lt;fascia-eta&gt;&lt;cod&gt;FE10&lt;/cod&gt;&lt;decod&gt;&lt;en&gt;60-64&lt;/en&gt;&lt;it&gt;60-64&lt;/it&gt;&lt;/decod&gt;&lt;/fascia-eta&gt;&lt;descrizione-ruolo-team&gt;&lt;en&gt;structural calculator&lt;/en&gt;&lt;it&gt;calcolatore strutturale&lt;/it&gt;&lt;/descrizione-ruolo-team&gt;&lt;/soggetto&gt;&lt;/team&gt;&lt;mercato&gt;&lt;area-geografica&gt;&lt;cod&gt;A4&lt;/cod&gt;&lt;decod&gt;&lt;en&gt;Italy&lt;/en&gt;&lt;it&gt;Italia&lt;/it&gt;&lt;/decod&gt;&lt;/area-geografica&gt;&lt;canale-di-vendita&gt;&lt;cod&gt;C1&lt;/cod&gt;&lt;decod&gt;&lt;en&gt;Directly&lt;/en&gt;&lt;it&gt;Direttamente&lt;/it&gt;&lt;/decod&gt;&lt;/canale-di-vendita&gt;&lt;/mercato&gt;&lt;business-model&gt;&lt;descrizione-business-model&gt;&lt;en&gt;The Italian real estate stock consists of over 29 million homes for 60 million residents; of these, about 10 million are built in the seismic areas most at risk: 1.4 million are located in zone 1 and about 9 million in zone 2. On the other hand, 8.5 million homes are located in zone 3 and 9.4 million, finally, in zone 4. Furthermore, the Italian residential building heritage tends to the old. The country's building and infrastructure capital have entered a cycle of growing obsolescence. Of the 12.2 million residential buildings surveyed by Istat, for example, 7.2 million (60%) were built before 1980; 5.2 million (42.5%) are over 50 years old. More than half of the homes - over 16 million - were built before 1970.&amp;#x0D;
+At least one third of the buildings should be adapted.&amp;#x0D;
+According to the estimates of the National Council of Engineers, a little more than 90 billion euros would be needed to secure the Italian residential assets; just over 50 could even be enough for the Civil Protection.&amp;#x0D;
+So we can estimate the total available market (TAM) at 70 billion euros (average of the two estimates mentioned above).&amp;#x0D;
+To estimate the achievable market (SAM), Italians' perception of seismic risk must be taken into account. From the analysis of the behavior of Italians, it appears that this risk is underestimated.&amp;#x0D;
+Proof of this is the incidence of anti-seismic renovations on the total renovations carried out by Italians in the two-year period 2015-2016: the buildings for which earthquake-resistant interventions were declared are just over 33,000, while the buildings for which renovations have been declared , in the year 2016 alone, there are almost 1.5 million.&amp;#x0D;
+In the period 2013-2016 just over 195 thousand anti-seismic interventions were carried out. The total amount of expenditure for this category of works was over 872 million euros.&amp;#x0D;
+For 2020, the A.N.C.E. foresees an increase of 1.5% for investments in extraordinary maintenance of the housing stock. The estimate takes into account, among other things, the impact on production levels of the interventions aimed at reducing the seismic risk related to the bonus earthquake.&amp;#x0D;
+Therefore, we can calculate the reference SAM as the product of the average expenditure per intervention and the number of interventions per year increased by 1.5%, that is just under 74.9 million euros.&amp;#x0D;
+These studies predate the health emergency due to COVID 19.&amp;#x0D;
+To determine the SOM (market actually obtainable) it was necessary to take into account the degree of market concentration and the competitive advantage that one thinks can be obtained with the LE.A.D.&amp;#x0D;
+The most innovative techniques, and closest to the proposed system, currently available on the market, are based on the use of Brad type hysteretic dissipators (Buckling Restrained Axial Damper).&amp;#x0D;
+This technique generally provides for the direct insertion of the devices within the structural mesh, these devices have considerable dimensions but having an operation that involves both traction and compression, for reasons of instability and bulk, they can only reach limited spans.&amp;#x0D;
+The peculiarity of the LE.AD system consists in the adoption of high elastic limit tie rods, which allow a containment of the dimensions of the bracing, acting only in traction, therefore having no problems of instability, so much so that it can be installed and moved on site by few people without the aid of special equipment, the weight of the appliance in fact does not exceed 25 kg, also to the advantage of the aesthetic-functional aspects, as the system is easily concealable, as well as being extremely simple and quick to set up works, with a substantial reduction both in the execution times of the works, and in the impact and invasiveness of the same on the existing structure and on the finishing of the building on which it is intervened.&amp;#x0D;
+Furthermore, the chaining system, which can be considered an extension of the traditional chain-head key system, allows to intervene on much wider spans than the BRAD system, being based exclusively on traction and binding, a mechanism that is free from twisting problems due to instability due to buckling.&amp;#x0D;
+This advantage can be quantified in a lower cost for the user, as well as greater flexibility in implementation and less invasiveness on the existing.&amp;#x0D;
+In the current practice of seismic improvement, about 85% of the costs are determined by the accessory interventions of restoration of the finishes and systems, costs that are considerably reduced by the application of the LE.AD system, as the sewing of the structures does not require invasive interventions on the building and most of the finishes and installations can be preserved.&amp;#x0D;
+The technological and functional advantage of the LE.A.D. will allow the company to overcome the technological barriers to entry to the reference market, since the system is highly innovative compared to systems already on the market.&amp;#x0D;
+Taking into account the advantageous position that it is presumed to be able to assume compared to competitors, we can p</t>
         </is>
       </c>
     </row>

</xml_diff>